<commit_message>
Modify schema condition to "keep" and all
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazym\Documents\Code\dissertation\build\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2AC10607-46AB-411C-A868-363265F1B791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D444940-3FDE-467C-AD24-B417C9CEBA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17280" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_properties" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="127">
   <si>
     <t>type</t>
   </si>
@@ -385,9 +385,6 @@
     <t>Blank for a lot of these</t>
   </si>
   <si>
-    <t>fixed_1_id</t>
-  </si>
-  <si>
     <t>avail_ptaddress</t>
   </si>
   <si>
@@ -398,6 +395,12 @@
   </si>
   <si>
     <t>derived</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>fixed</t>
   </si>
 </sst>
 </file>
@@ -1270,18 +1273,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
   <dimension ref="A1:I53"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.453125" customWidth="1"/>
-    <col min="2" max="2" width="38.7265625" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" customWidth="1"/>
-    <col min="4" max="4" width="38.26953125" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>105</v>
@@ -1305,7 +1308,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1322,7 +1325,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -1331,7 +1334,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1348,13 +1351,13 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1377,7 +1380,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1397,7 +1400,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1414,7 +1417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1448,7 +1451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1465,7 +1468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1482,7 +1485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1499,7 +1502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1516,7 +1519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1533,7 +1536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -1550,7 +1553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -1567,7 +1570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1584,7 +1587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1601,7 +1604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -1618,7 +1621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -1635,7 +1638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -1652,7 +1655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>2</v>
       </c>
@@ -1669,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -1686,7 +1689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -1706,7 +1709,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -1723,7 +1726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -1740,7 +1743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -1760,7 +1763,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -1780,7 +1783,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -1797,7 +1800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G29" t="b">
         <v>1</v>
@@ -1823,7 +1826,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -1840,13 +1843,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G30" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -1863,7 +1866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -1907,7 +1910,7 @@
       </c>
       <c r="I33" s="3"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -1925,7 +1928,7 @@
       </c>
       <c r="I34" s="3"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -1943,7 +1946,7 @@
       </c>
       <c r="I35" s="3"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>2</v>
       </c>
@@ -1961,7 +1964,7 @@
       </c>
       <c r="I36" s="3"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -1979,7 +1982,7 @@
       </c>
       <c r="I37" s="3"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -1997,7 +2000,7 @@
       </c>
       <c r="I38" s="3"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -2015,7 +2018,7 @@
       </c>
       <c r="I39" s="3"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -2033,7 +2036,7 @@
       </c>
       <c r="I40" s="3"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -2051,7 +2054,7 @@
       </c>
       <c r="I41" s="3"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -2069,7 +2072,7 @@
       </c>
       <c r="I42" s="3"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>2</v>
       </c>
@@ -2087,7 +2090,7 @@
       </c>
       <c r="I43" s="3"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -2105,7 +2108,7 @@
       </c>
       <c r="I44" s="3"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>2</v>
       </c>
@@ -2123,7 +2126,7 @@
       </c>
       <c r="I45" s="3"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -2141,7 +2144,7 @@
       </c>
       <c r="I46" s="3"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -2159,7 +2162,7 @@
       </c>
       <c r="I47" s="3"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2177,7 +2180,7 @@
       </c>
       <c r="I48" s="3"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -2194,7 +2197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -2211,12 +2214,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>125</v>
-      </c>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C51" t="s">
         <v>98</v>
@@ -2224,16 +2224,16 @@
       <c r="E51" t="b">
         <v>1</v>
       </c>
+      <c r="F51" t="s">
+        <v>124</v>
+      </c>
       <c r="H51" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>125</v>
-      </c>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C52" t="s">
         <v>98</v>
@@ -2241,11 +2241,11 @@
       <c r="E52" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>125</v>
-      </c>
+      <c r="F52" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>110</v>
       </c>
@@ -2254,6 +2254,9 @@
       </c>
       <c r="E53" t="b">
         <v>1</v>
+      </c>
+      <c r="F53" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Some really great file parsing
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F12743-0D31-4B50-9E31-9DA218EB94E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E14081-2C40-4CB5-93EE-A82CB7EFB8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="133">
   <si>
     <t>type</t>
   </si>
@@ -421,6 +421,18 @@
   <si>
     <t>Strategy,  organization and policy
 Strategy, organization and policy</t>
+  </si>
+  <si>
+    <t>file_code</t>
+  </si>
+  <si>
+    <t>str</t>
+  </si>
+  <si>
+    <t>From the filepaths</t>
+  </si>
+  <si>
+    <t>industry_code</t>
   </si>
 </sst>
 </file>
@@ -1295,7 +1307,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -2071,6 +2083,12 @@
       <c r="D49" t="s">
         <v>94</v>
       </c>
+      <c r="E49" t="s">
+        <v>122</v>
+      </c>
+      <c r="F49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -2084,6 +2102,12 @@
       </c>
       <c r="D50" t="s">
         <v>97</v>
+      </c>
+      <c r="E50" t="s">
+        <v>122</v>
+      </c>
+      <c r="F50" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -2134,6 +2158,34 @@
       </c>
       <c r="E54" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>132</v>
+      </c>
+      <c r="C55" t="s">
+        <v>130</v>
+      </c>
+      <c r="E55" t="s">
+        <v>120</v>
+      </c>
+      <c r="G55" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>129</v>
+      </c>
+      <c r="C56" t="s">
+        <v>130</v>
+      </c>
+      <c r="E56" t="s">
+        <v>120</v>
+      </c>
+      <c r="G56" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Huge progress entering in 2 tables
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E14081-2C40-4CB5-93EE-A82CB7EFB8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA18877-65CD-450F-ADAD-1FE32DCB473D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
+    <workbookView xWindow="-38505" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_properties" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="134">
   <si>
     <t>type</t>
   </si>
@@ -323,9 +323,6 @@
     <t>no_of_available_years</t>
   </si>
   <si>
-    <t>int32</t>
-  </si>
-  <si>
     <t>No of available years</t>
   </si>
   <si>
@@ -362,9 +359,6 @@
     <t>is_public</t>
   </si>
   <si>
-    <t>primary_tra</t>
-  </si>
-  <si>
     <t>I. core</t>
   </si>
   <si>
@@ -378,9 +372,6 @@
   </si>
   <si>
     <t>SIC was updated in 2007. UK SIC: 2026 - Office for National Statistics</t>
-  </si>
-  <si>
-    <t>same as company_name for most, missing for others</t>
   </si>
   <si>
     <t>Formerly known as …' for a few</t>
@@ -433,6 +424,18 @@
   </si>
   <si>
     <t>industry_code</t>
+  </si>
+  <si>
+    <t>same as company_name for most, missing for others. Lars calls it 'company_name_B</t>
+  </si>
+  <si>
+    <t>has_company_branch_mismatch</t>
+  </si>
+  <si>
+    <t>primary trading address missing</t>
+  </si>
+  <si>
+    <t>int64</t>
   </si>
 </sst>
 </file>
@@ -1307,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1318,10 +1321,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -1330,13 +1333,13 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1353,18 +1356,18 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -1376,7 +1379,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -1395,11 +1398,14 @@
       <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="b">
+      <c r="E4" t="s">
+        <v>119</v>
+      </c>
+      <c r="F4" t="b">
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1416,7 +1422,7 @@
         <v>11</v>
       </c>
       <c r="H5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1430,7 +1436,7 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1444,7 +1450,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1458,7 +1464,7 @@
         <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1472,7 +1478,7 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1486,7 +1492,7 @@
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1670,8 +1676,14 @@
       <c r="D23" t="s">
         <v>42</v>
       </c>
+      <c r="E23" t="s">
+        <v>119</v>
+      </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
       <c r="H23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1687,6 +1699,12 @@
       <c r="D24" t="s">
         <v>44</v>
       </c>
+      <c r="E24" t="s">
+        <v>119</v>
+      </c>
+      <c r="F24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1701,6 +1719,12 @@
       <c r="D25" t="s">
         <v>46</v>
       </c>
+      <c r="E25" t="s">
+        <v>119</v>
+      </c>
+      <c r="F25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1710,13 +1734,13 @@
         <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
         <v>48</v>
       </c>
       <c r="G26" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1732,8 +1756,14 @@
       <c r="D27" t="s">
         <v>50</v>
       </c>
+      <c r="E27" t="s">
+        <v>119</v>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
       <c r="G27" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1758,19 +1788,19 @@
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
       <c r="D29" t="s">
         <v>54</v>
       </c>
       <c r="E29" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F29" t="b">
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1787,7 +1817,7 @@
         <v>56</v>
       </c>
       <c r="E30" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -1824,10 +1854,10 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1931,7 +1961,7 @@
         <v>4</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H39" s="3"/>
     </row>
@@ -2084,7 +2114,7 @@
         <v>94</v>
       </c>
       <c r="E49" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F49" t="b">
         <v>1</v>
@@ -2098,13 +2128,13 @@
         <v>95</v>
       </c>
       <c r="C50" t="s">
+        <v>133</v>
+      </c>
+      <c r="D50" t="s">
         <v>96</v>
       </c>
-      <c r="D50" t="s">
-        <v>97</v>
-      </c>
       <c r="E50" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F50" t="b">
         <v>1</v>
@@ -2112,80 +2142,91 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C51" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E51" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G51" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C52" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E52" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E53" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C54" t="s">
-        <v>96</v>
-      </c>
-      <c r="D54" t="s">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="E54" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C55" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E55" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G55" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C56" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E56" t="s">
+        <v>117</v>
+      </c>
+      <c r="G56" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" t="s">
+        <v>133</v>
+      </c>
+      <c r="D57" t="s">
+        <v>122</v>
+      </c>
+      <c r="E57" t="s">
         <v>120</v>
-      </c>
-      <c r="G56" t="s">
-        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Begin work on processing yearly data
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA18877-65CD-450F-ADAD-1FE32DCB473D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3E6696-8AE4-4535-84EB-1A2448FB5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38505" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_properties" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="236">
   <si>
     <t>type</t>
   </si>
@@ -436,6 +436,348 @@
   </si>
   <si>
     <t>int64</t>
+  </si>
+  <si>
+    <t>a2_key_finance</t>
+  </si>
+  <si>
+    <t>consolidated</t>
+  </si>
+  <si>
+    <t>Cons./Uncons.</t>
+  </si>
+  <si>
+    <t>turnover</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>Turnoverth GBP</t>
+  </si>
+  <si>
+    <t>shareholders_funds</t>
+  </si>
+  <si>
+    <t>Shareholders Funds
+th GBP</t>
+  </si>
+  <si>
+    <t>Profit (Loss) before Taxation
+th GBP</t>
+  </si>
+  <si>
+    <t>profit_loss_pretax</t>
+  </si>
+  <si>
+    <t>employees</t>
+  </si>
+  <si>
+    <t>fint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of employees
+</t>
+  </si>
+  <si>
+    <t>Number of employees</t>
+  </si>
+  <si>
+    <t>Tangible Assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Land &amp; Buildings
+th GBP</t>
+  </si>
+  <si>
+    <t>Freehold Land
+th GBP</t>
+  </si>
+  <si>
+    <t>Leasehold Land
+th GBP</t>
+  </si>
+  <si>
+    <t>Fixtures &amp; Fittings
+th GBP</t>
+  </si>
+  <si>
+    <t>Plant &amp; Vehicles
+th GBP</t>
+  </si>
+  <si>
+    <t>Plant
+th GBP</t>
+  </si>
+  <si>
+    <t>Vehicles
+th GBP</t>
+  </si>
+  <si>
+    <t>Other Fixed Assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Intangible Assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Investments &amp; other fixed assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Fixed Assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Current Liabilities
+th GBP</t>
+  </si>
+  <si>
+    <t>Total Assets
+th GBP</t>
+  </si>
+  <si>
+    <t>Long Term Liabilities
+th GBP</t>
+  </si>
+  <si>
+    <t>a3_assets</t>
+  </si>
+  <si>
+    <t>tangibles</t>
+  </si>
+  <si>
+    <t>intangibles</t>
+  </si>
+  <si>
+    <t>tangibles_land_and_buildings</t>
+  </si>
+  <si>
+    <t>tangibles_land_freehold</t>
+  </si>
+  <si>
+    <t>tangibles_land_leasehold</t>
+  </si>
+  <si>
+    <t>tangibles_plant_and_vehicles</t>
+  </si>
+  <si>
+    <t>tangibles_plant</t>
+  </si>
+  <si>
+    <t>tangibles_vehicles</t>
+  </si>
+  <si>
+    <t>investments_other</t>
+  </si>
+  <si>
+    <t>liabilities</t>
+  </si>
+  <si>
+    <t>total_assets</t>
+  </si>
+  <si>
+    <t>liabilites_lt</t>
+  </si>
+  <si>
+    <t>fixed_other</t>
+  </si>
+  <si>
+    <t>fixed_total</t>
+  </si>
+  <si>
+    <t>Turnover
+th GBP</t>
+  </si>
+  <si>
+    <t>Cost of Sales
+th GBP</t>
+  </si>
+  <si>
+    <t>Administration Expenses
+th GBP</t>
+  </si>
+  <si>
+    <t>Interest Paid
+th GBP</t>
+  </si>
+  <si>
+    <t>Profit (Loss) before Tax
+th GBP</t>
+  </si>
+  <si>
+    <t>Taxation
+th GBP</t>
+  </si>
+  <si>
+    <t>Dividends (Distributable profit)
+th GBP</t>
+  </si>
+  <si>
+    <t>Depreciation
+th GBP</t>
+  </si>
+  <si>
+    <t>Research &amp; Development
+th GBP</t>
+  </si>
+  <si>
+    <t>Remuneration
+th GBP</t>
+  </si>
+  <si>
+    <t>Wages &amp; Salaries
+th GBP</t>
+  </si>
+  <si>
+    <t>Social Security Costs
+th GBP</t>
+  </si>
+  <si>
+    <t>Pension Costs
+th GBP</t>
+  </si>
+  <si>
+    <t>Other Staff Costs
+th GBP</t>
+  </si>
+  <si>
+    <t>Directors' Remuneration
+th GBP</t>
+  </si>
+  <si>
+    <t>EBITDA
+th GBP</t>
+  </si>
+  <si>
+    <t>a4_profits</t>
+  </si>
+  <si>
+    <t>tangibles_fixt_fit</t>
+  </si>
+  <si>
+    <t>cos</t>
+  </si>
+  <si>
+    <t>tax</t>
+  </si>
+  <si>
+    <t>admin_expenses</t>
+  </si>
+  <si>
+    <t>interest_paid</t>
+  </si>
+  <si>
+    <t>turnover2</t>
+  </si>
+  <si>
+    <t>profit_loss_pretax2</t>
+  </si>
+  <si>
+    <t>dividends</t>
+  </si>
+  <si>
+    <t>depreciation</t>
+  </si>
+  <si>
+    <t>r_and_d</t>
+  </si>
+  <si>
+    <t>wages</t>
+  </si>
+  <si>
+    <t>social_security_costs</t>
+  </si>
+  <si>
+    <t>pensions_costs</t>
+  </si>
+  <si>
+    <t>other_staff_costs</t>
+  </si>
+  <si>
+    <t>renumeration_directors</t>
+  </si>
+  <si>
+    <t>remuneration_employees</t>
+  </si>
+  <si>
+    <t>employees2</t>
+  </si>
+  <si>
+    <t>ebitda</t>
+  </si>
+  <si>
+    <t>Credit score</t>
+  </si>
+  <si>
+    <t>Credit score date</t>
+  </si>
+  <si>
+    <t>Credit score indicator</t>
+  </si>
+  <si>
+    <t>Likelihood of failure
+%</t>
+  </si>
+  <si>
+    <t>Credit limit
+GBP</t>
+  </si>
+  <si>
+    <t>Previous credit score</t>
+  </si>
+  <si>
+    <t>Previous credit score indicator</t>
+  </si>
+  <si>
+    <t>Ultimate owner</t>
+  </si>
+  <si>
+    <t>No of companies in corporate group</t>
+  </si>
+  <si>
+    <t>Entity type</t>
+  </si>
+  <si>
+    <t>credit_score</t>
+  </si>
+  <si>
+    <t>entity_type</t>
+  </si>
+  <si>
+    <t>credit_score_date</t>
+  </si>
+  <si>
+    <t>credit_score_indicator</t>
+  </si>
+  <si>
+    <t>likelihood_failure</t>
+  </si>
+  <si>
+    <t>credit_limit</t>
+  </si>
+  <si>
+    <t>credit_score_prev</t>
+  </si>
+  <si>
+    <t>credit_score_indicator_prev</t>
+  </si>
+  <si>
+    <t>guo</t>
+  </si>
+  <si>
+    <t>guo_nb</t>
+  </si>
+  <si>
+    <t>a5_misc</t>
+  </si>
+  <si>
+    <t>global ultimate owner</t>
+  </si>
+  <si>
+    <t>number of other firms in the same group</t>
   </si>
 </sst>
 </file>
@@ -925,15 +1267,22 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1310,13 +1659,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" customWidth="1"/>
     <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="38.28515625" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1332,7 +1682,7 @@
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1355,7 +1705,7 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F2" t="b">
@@ -1378,7 +1728,7 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="7" t="s">
         <v>118</v>
       </c>
       <c r="F3" t="b">
@@ -1398,11 +1748,8 @@
       <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="7" t="s">
         <v>119</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
       </c>
       <c r="G4" t="s">
         <v>106</v>
@@ -1676,7 +2023,7 @@
       <c r="D23" t="s">
         <v>42</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F23" t="b">
@@ -1699,7 +2046,7 @@
       <c r="D24" t="s">
         <v>44</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F24" t="b">
@@ -1719,7 +2066,7 @@
       <c r="D25" t="s">
         <v>46</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F25" t="b">
@@ -1756,7 +2103,7 @@
       <c r="D27" t="s">
         <v>50</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F27" t="b">
@@ -1793,7 +2140,7 @@
       <c r="D29" t="s">
         <v>54</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F29" t="b">
@@ -1816,7 +2163,7 @@
       <c r="D30" t="s">
         <v>56</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F30" t="b">
@@ -1850,13 +2197,13 @@
       <c r="D32" t="s">
         <v>60</v>
       </c>
-      <c r="E32" t="b">
+      <c r="E32" s="7" t="b">
         <v>0</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="4" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1873,7 +2220,7 @@
       <c r="D33" t="s">
         <v>62</v>
       </c>
-      <c r="H33" s="3"/>
+      <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -1888,7 +2235,7 @@
       <c r="D34" t="s">
         <v>64</v>
       </c>
-      <c r="H34" s="3"/>
+      <c r="H34" s="4"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -1903,7 +2250,7 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-      <c r="H35" s="3"/>
+      <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
@@ -1918,7 +2265,7 @@
       <c r="D36" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="3"/>
+      <c r="H36" s="4"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -1933,7 +2280,7 @@
       <c r="D37" t="s">
         <v>70</v>
       </c>
-      <c r="H37" s="3"/>
+      <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
@@ -1948,7 +2295,7 @@
       <c r="D38" t="s">
         <v>72</v>
       </c>
-      <c r="H38" s="3"/>
+      <c r="H38" s="4"/>
     </row>
     <row r="39" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -1960,10 +2307,10 @@
       <c r="C39" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="4"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -1978,7 +2325,7 @@
       <c r="D40" t="s">
         <v>75</v>
       </c>
-      <c r="H40" s="3"/>
+      <c r="H40" s="4"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -1993,7 +2340,7 @@
       <c r="D41" t="s">
         <v>77</v>
       </c>
-      <c r="H41" s="3"/>
+      <c r="H41" s="4"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
@@ -2008,7 +2355,7 @@
       <c r="D42" t="s">
         <v>79</v>
       </c>
-      <c r="H42" s="3"/>
+      <c r="H42" s="4"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
@@ -2023,7 +2370,7 @@
       <c r="D43" t="s">
         <v>81</v>
       </c>
-      <c r="H43" s="3"/>
+      <c r="H43" s="4"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
@@ -2038,7 +2385,7 @@
       <c r="D44" t="s">
         <v>83</v>
       </c>
-      <c r="H44" s="3"/>
+      <c r="H44" s="4"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -2053,7 +2400,7 @@
       <c r="D45" t="s">
         <v>85</v>
       </c>
-      <c r="H45" s="3"/>
+      <c r="H45" s="4"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -2068,7 +2415,7 @@
       <c r="D46" t="s">
         <v>87</v>
       </c>
-      <c r="H46" s="3"/>
+      <c r="H46" s="4"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
@@ -2083,7 +2430,7 @@
       <c r="D47" t="s">
         <v>89</v>
       </c>
-      <c r="H47" s="3"/>
+      <c r="H47" s="4"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
@@ -2098,7 +2445,7 @@
       <c r="D48" t="s">
         <v>91</v>
       </c>
-      <c r="H48" s="3"/>
+      <c r="H48" s="4"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -2113,7 +2460,7 @@
       <c r="D49" t="s">
         <v>94</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F49" t="b">
@@ -2133,7 +2480,7 @@
       <c r="D50" t="s">
         <v>96</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="7" t="s">
         <v>119</v>
       </c>
       <c r="F50" t="b">
@@ -2147,7 +2494,7 @@
       <c r="C51" t="s">
         <v>97</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="7" t="s">
         <v>117</v>
       </c>
       <c r="G51" t="s">
@@ -2161,7 +2508,7 @@
       <c r="C52" t="s">
         <v>97</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" s="7" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2172,7 +2519,7 @@
       <c r="C53" t="s">
         <v>97</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="7" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2183,7 +2530,7 @@
       <c r="C54" t="s">
         <v>97</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E54" s="7" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2194,7 +2541,7 @@
       <c r="C55" t="s">
         <v>127</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E55" s="7" t="s">
         <v>117</v>
       </c>
       <c r="G55" t="s">
@@ -2208,7 +2555,7 @@
       <c r="C56" t="s">
         <v>127</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" s="7" t="s">
         <v>117</v>
       </c>
       <c r="G56" t="s">
@@ -2225,8 +2572,804 @@
       <c r="D57" t="s">
         <v>122</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E57" s="7" t="s">
         <v>120</v>
+      </c>
+      <c r="F57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>134</v>
+      </c>
+      <c r="B58" t="s">
+        <v>135</v>
+      </c>
+      <c r="C58" t="s">
+        <v>97</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>134</v>
+      </c>
+      <c r="B59" t="s">
+        <v>137</v>
+      </c>
+      <c r="C59" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>134</v>
+      </c>
+      <c r="B60" t="s">
+        <v>140</v>
+      </c>
+      <c r="C60" t="s">
+        <v>138</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>134</v>
+      </c>
+      <c r="B61" t="s">
+        <v>143</v>
+      </c>
+      <c r="C61" t="s">
+        <v>138</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>134</v>
+      </c>
+      <c r="B62" t="s">
+        <v>144</v>
+      </c>
+      <c r="C62" t="s">
+        <v>145</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>163</v>
+      </c>
+      <c r="B63" t="s">
+        <v>164</v>
+      </c>
+      <c r="C63" t="s">
+        <v>138</v>
+      </c>
+      <c r="D63" t="s">
+        <v>148</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>163</v>
+      </c>
+      <c r="B64" t="s">
+        <v>166</v>
+      </c>
+      <c r="C64" t="s">
+        <v>138</v>
+      </c>
+      <c r="D64" t="s">
+        <v>149</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>163</v>
+      </c>
+      <c r="B65" t="s">
+        <v>167</v>
+      </c>
+      <c r="C65" t="s">
+        <v>138</v>
+      </c>
+      <c r="D65" t="s">
+        <v>150</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>163</v>
+      </c>
+      <c r="B66" t="s">
+        <v>168</v>
+      </c>
+      <c r="C66" t="s">
+        <v>138</v>
+      </c>
+      <c r="D66" t="s">
+        <v>151</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>163</v>
+      </c>
+      <c r="B67" t="s">
+        <v>195</v>
+      </c>
+      <c r="C67" t="s">
+        <v>138</v>
+      </c>
+      <c r="D67" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>163</v>
+      </c>
+      <c r="B68" t="s">
+        <v>169</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+      <c r="D68" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>163</v>
+      </c>
+      <c r="B69" t="s">
+        <v>170</v>
+      </c>
+      <c r="C69" t="s">
+        <v>138</v>
+      </c>
+      <c r="D69" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>163</v>
+      </c>
+      <c r="B70" t="s">
+        <v>171</v>
+      </c>
+      <c r="C70" t="s">
+        <v>138</v>
+      </c>
+      <c r="D70" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>163</v>
+      </c>
+      <c r="B71" t="s">
+        <v>176</v>
+      </c>
+      <c r="C71" t="s">
+        <v>138</v>
+      </c>
+      <c r="D71" t="s">
+        <v>156</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>163</v>
+      </c>
+      <c r="B72" t="s">
+        <v>165</v>
+      </c>
+      <c r="C72" t="s">
+        <v>138</v>
+      </c>
+      <c r="D72" t="s">
+        <v>157</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>163</v>
+      </c>
+      <c r="B73" t="s">
+        <v>172</v>
+      </c>
+      <c r="C73" t="s">
+        <v>138</v>
+      </c>
+      <c r="D73" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>163</v>
+      </c>
+      <c r="B74" t="s">
+        <v>177</v>
+      </c>
+      <c r="C74" t="s">
+        <v>138</v>
+      </c>
+      <c r="D74" t="s">
+        <v>159</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>163</v>
+      </c>
+      <c r="B75" t="s">
+        <v>173</v>
+      </c>
+      <c r="C75" t="s">
+        <v>138</v>
+      </c>
+      <c r="D75" t="s">
+        <v>160</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>163</v>
+      </c>
+      <c r="B76" t="s">
+        <v>174</v>
+      </c>
+      <c r="C76" t="s">
+        <v>138</v>
+      </c>
+      <c r="D76" t="s">
+        <v>161</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>163</v>
+      </c>
+      <c r="B77" t="s">
+        <v>175</v>
+      </c>
+      <c r="C77" t="s">
+        <v>138</v>
+      </c>
+      <c r="D77" t="s">
+        <v>162</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>194</v>
+      </c>
+      <c r="B78" t="s">
+        <v>200</v>
+      </c>
+      <c r="C78" t="s">
+        <v>138</v>
+      </c>
+      <c r="D78" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>194</v>
+      </c>
+      <c r="B79" t="s">
+        <v>196</v>
+      </c>
+      <c r="C79" t="s">
+        <v>138</v>
+      </c>
+      <c r="D79" t="s">
+        <v>179</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>194</v>
+      </c>
+      <c r="B80" t="s">
+        <v>198</v>
+      </c>
+      <c r="C80" t="s">
+        <v>138</v>
+      </c>
+      <c r="D80" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>194</v>
+      </c>
+      <c r="B81" t="s">
+        <v>199</v>
+      </c>
+      <c r="C81" t="s">
+        <v>138</v>
+      </c>
+      <c r="D81" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>194</v>
+      </c>
+      <c r="B82" t="s">
+        <v>201</v>
+      </c>
+      <c r="C82" t="s">
+        <v>138</v>
+      </c>
+      <c r="D82" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>194</v>
+      </c>
+      <c r="B83" t="s">
+        <v>197</v>
+      </c>
+      <c r="C83" t="s">
+        <v>138</v>
+      </c>
+      <c r="D83" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>194</v>
+      </c>
+      <c r="B84" t="s">
+        <v>202</v>
+      </c>
+      <c r="C84" t="s">
+        <v>138</v>
+      </c>
+      <c r="D84" t="s">
+        <v>184</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F84" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>194</v>
+      </c>
+      <c r="B85" t="s">
+        <v>203</v>
+      </c>
+      <c r="C85" t="s">
+        <v>138</v>
+      </c>
+      <c r="D85" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>194</v>
+      </c>
+      <c r="B86" t="s">
+        <v>204</v>
+      </c>
+      <c r="C86" t="s">
+        <v>138</v>
+      </c>
+      <c r="D86" t="s">
+        <v>186</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F86" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>194</v>
+      </c>
+      <c r="B87" t="s">
+        <v>210</v>
+      </c>
+      <c r="C87" t="s">
+        <v>138</v>
+      </c>
+      <c r="D87" t="s">
+        <v>187</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>194</v>
+      </c>
+      <c r="B88" t="s">
+        <v>205</v>
+      </c>
+      <c r="C88" t="s">
+        <v>138</v>
+      </c>
+      <c r="D88" t="s">
+        <v>188</v>
+      </c>
+      <c r="E88" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>194</v>
+      </c>
+      <c r="B89" t="s">
+        <v>206</v>
+      </c>
+      <c r="C89" t="s">
+        <v>138</v>
+      </c>
+      <c r="D89" t="s">
+        <v>189</v>
+      </c>
+      <c r="E89" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F89" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>194</v>
+      </c>
+      <c r="B90" t="s">
+        <v>207</v>
+      </c>
+      <c r="C90" t="s">
+        <v>138</v>
+      </c>
+      <c r="D90" t="s">
+        <v>190</v>
+      </c>
+      <c r="E90" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F90" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>194</v>
+      </c>
+      <c r="B91" t="s">
+        <v>208</v>
+      </c>
+      <c r="C91" t="s">
+        <v>138</v>
+      </c>
+      <c r="D91" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>194</v>
+      </c>
+      <c r="B92" t="s">
+        <v>209</v>
+      </c>
+      <c r="C92" t="s">
+        <v>138</v>
+      </c>
+      <c r="D92" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>194</v>
+      </c>
+      <c r="B93" t="s">
+        <v>211</v>
+      </c>
+      <c r="C93" t="s">
+        <v>138</v>
+      </c>
+      <c r="D93" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>194</v>
+      </c>
+      <c r="B94" t="s">
+        <v>212</v>
+      </c>
+      <c r="C94" t="s">
+        <v>138</v>
+      </c>
+      <c r="D94" t="s">
+        <v>193</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F94" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>233</v>
+      </c>
+      <c r="B95" t="s">
+        <v>223</v>
+      </c>
+      <c r="C95" t="s">
+        <v>133</v>
+      </c>
+      <c r="D95" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>233</v>
+      </c>
+      <c r="B96" t="s">
+        <v>225</v>
+      </c>
+      <c r="C96" t="s">
+        <v>93</v>
+      </c>
+      <c r="D96" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>233</v>
+      </c>
+      <c r="B97" t="s">
+        <v>226</v>
+      </c>
+      <c r="C97" t="s">
+        <v>4</v>
+      </c>
+      <c r="D97" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>233</v>
+      </c>
+      <c r="B98" t="s">
+        <v>227</v>
+      </c>
+      <c r="C98" t="s">
+        <v>138</v>
+      </c>
+      <c r="D98" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>233</v>
+      </c>
+      <c r="B99" t="s">
+        <v>228</v>
+      </c>
+      <c r="C99" t="s">
+        <v>133</v>
+      </c>
+      <c r="D99" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>233</v>
+      </c>
+      <c r="B100" t="s">
+        <v>229</v>
+      </c>
+      <c r="C100" t="s">
+        <v>133</v>
+      </c>
+      <c r="D100" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>233</v>
+      </c>
+      <c r="B101" t="s">
+        <v>230</v>
+      </c>
+      <c r="C101" t="s">
+        <v>4</v>
+      </c>
+      <c r="D101" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>233</v>
+      </c>
+      <c r="B102" t="s">
+        <v>231</v>
+      </c>
+      <c r="C102" t="s">
+        <v>4</v>
+      </c>
+      <c r="D102" t="s">
+        <v>220</v>
+      </c>
+      <c r="E102" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G102" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>233</v>
+      </c>
+      <c r="B103" t="s">
+        <v>232</v>
+      </c>
+      <c r="C103" t="s">
+        <v>133</v>
+      </c>
+      <c r="D103" t="s">
+        <v>221</v>
+      </c>
+      <c r="E103" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G103" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>233</v>
+      </c>
+      <c r="B104" t="s">
+        <v>224</v>
+      </c>
+      <c r="C104" t="s">
+        <v>4</v>
+      </c>
+      <c r="D104" t="s">
+        <v>222</v>
+      </c>
+      <c r="E104" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modifications to the raw_properties table
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E3E6696-8AE4-4535-84EB-1A2448FB5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4BC391-9E29-4809-85E3-5D76DBDB0FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="237">
   <si>
     <t>type</t>
   </si>
@@ -473,9 +473,6 @@
     <t>employees</t>
   </si>
   <si>
-    <t>fint</t>
-  </si>
-  <si>
     <t xml:space="preserve">Number of employees
 </t>
   </si>
@@ -778,6 +775,12 @@
   </si>
   <si>
     <t>number of other firms in the same group</t>
+  </si>
+  <si>
+    <t>fame_key</t>
+  </si>
+  <si>
+    <t>2 special rows that index the below</t>
   </si>
 </sst>
 </file>
@@ -926,7 +929,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1106,6 +1109,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1267,7 +1276,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1284,6 +1293,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1659,7 +1669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -2563,37 +2573,34 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B57" t="s">
-        <v>121</v>
+      <c r="B57" s="8" t="s">
+        <v>235</v>
       </c>
       <c r="C57" t="s">
-        <v>133</v>
-      </c>
-      <c r="D57" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F57" t="b">
-        <v>1</v>
+      <c r="G57" s="1" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>134</v>
-      </c>
-      <c r="B58" t="s">
-        <v>135</v>
+      <c r="B58" s="8" t="s">
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>97</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
+      </c>
+      <c r="D58" t="s">
+        <v>122</v>
       </c>
       <c r="E58" s="7" t="s">
         <v>120</v>
+      </c>
+      <c r="F58" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -2601,19 +2608,16 @@
         <v>134</v>
       </c>
       <c r="B59" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C59" t="s">
-        <v>138</v>
+        <v>97</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="F59" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -2621,13 +2625,13 @@
         <v>134</v>
       </c>
       <c r="B60" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C60" t="s">
         <v>138</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E60" s="7" t="s">
         <v>120</v>
@@ -2641,13 +2645,13 @@
         <v>134</v>
       </c>
       <c r="B61" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C61" t="s">
         <v>138</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>120</v>
@@ -2661,13 +2665,13 @@
         <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C62" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>120</v>
@@ -2678,16 +2682,16 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
       <c r="B63" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
       <c r="C63" t="s">
-        <v>138</v>
-      </c>
-      <c r="D63" t="s">
-        <v>148</v>
+        <v>133</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="E63" s="7" t="s">
         <v>120</v>
@@ -2698,33 +2702,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>162</v>
+      </c>
+      <c r="B64" t="s">
         <v>163</v>
       </c>
-      <c r="B64" t="s">
-        <v>166</v>
-      </c>
       <c r="C64" t="s">
         <v>138</v>
       </c>
       <c r="D64" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>120</v>
       </c>
+      <c r="F64" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B65" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C65" t="s">
         <v>138</v>
       </c>
       <c r="D65" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>120</v>
@@ -2732,16 +2739,16 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B66" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C66" t="s">
         <v>138</v>
       </c>
       <c r="D66" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>120</v>
@@ -2749,92 +2756,89 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
       <c r="C67" t="s">
         <v>138</v>
       </c>
       <c r="D67" t="s">
-        <v>152</v>
+        <v>150</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="C68" t="s">
         <v>138</v>
       </c>
       <c r="D68" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B69" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C69" t="s">
         <v>138</v>
       </c>
       <c r="D69" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B70" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C70" t="s">
         <v>138</v>
       </c>
       <c r="D70" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B71" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C71" t="s">
         <v>138</v>
       </c>
       <c r="D71" t="s">
-        <v>156</v>
-      </c>
-      <c r="E71" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F71" t="b">
-        <v>1</v>
+        <v>154</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B72" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="C72" t="s">
         <v>138</v>
       </c>
       <c r="D72" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>120</v>
@@ -2845,87 +2849,87 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B73" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C73" t="s">
         <v>138</v>
       </c>
       <c r="D73" t="s">
-        <v>158</v>
+        <v>156</v>
+      </c>
+      <c r="E73" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F73" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B74" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C74" t="s">
         <v>138</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
-      </c>
-      <c r="E74" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F74" t="b">
-        <v>1</v>
+        <v>157</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B75" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C75" t="s">
         <v>138</v>
       </c>
       <c r="D75" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>120</v>
       </c>
+      <c r="F75" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B76" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C76" t="s">
         <v>138</v>
       </c>
       <c r="D76" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E76" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F76" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B77" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C77" t="s">
         <v>138</v>
       </c>
       <c r="D77" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E77" s="7" t="s">
         <v>120</v>
@@ -2936,197 +2940,197 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="B78" t="s">
-        <v>200</v>
+        <v>174</v>
       </c>
       <c r="C78" t="s">
         <v>138</v>
       </c>
       <c r="D78" t="s">
-        <v>178</v>
+        <v>161</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F78" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B79" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C79" t="s">
         <v>138</v>
       </c>
       <c r="D79" t="s">
-        <v>179</v>
-      </c>
-      <c r="E79" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F79" t="b">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B80" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C80" t="s">
         <v>138</v>
       </c>
       <c r="D80" t="s">
-        <v>180</v>
+        <v>178</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F80" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B81" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C81" t="s">
         <v>138</v>
       </c>
       <c r="D81" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B82" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C82" t="s">
         <v>138</v>
       </c>
       <c r="D82" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B83" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C83" t="s">
         <v>138</v>
       </c>
       <c r="D83" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B84" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C84" t="s">
         <v>138</v>
       </c>
       <c r="D84" t="s">
-        <v>184</v>
-      </c>
-      <c r="E84" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F84" t="b">
-        <v>1</v>
+        <v>182</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B85" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C85" t="s">
         <v>138</v>
       </c>
       <c r="D85" t="s">
-        <v>185</v>
+        <v>183</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F85" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B86" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C86" t="s">
         <v>138</v>
       </c>
       <c r="D86" t="s">
-        <v>186</v>
-      </c>
-      <c r="E86" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F86" t="b">
-        <v>1</v>
+        <v>184</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B87" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C87" t="s">
         <v>138</v>
       </c>
       <c r="D87" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>120</v>
       </c>
+      <c r="F87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B88" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C88" t="s">
         <v>138</v>
       </c>
       <c r="D88" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="F88" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B89" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C89" t="s">
         <v>138</v>
       </c>
       <c r="D89" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>120</v>
@@ -3137,16 +3141,16 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B90" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C90" t="s">
         <v>138</v>
       </c>
       <c r="D90" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E90" s="7" t="s">
         <v>120</v>
@@ -3157,218 +3161,238 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B91" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C91" t="s">
         <v>138</v>
       </c>
       <c r="D91" t="s">
-        <v>191</v>
+        <v>189</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F91" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B92" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C92" t="s">
         <v>138</v>
       </c>
       <c r="D92" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B93" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C93" t="s">
         <v>138</v>
       </c>
       <c r="D93" t="s">
-        <v>146</v>
+        <v>191</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B94" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C94" t="s">
         <v>138</v>
       </c>
       <c r="D94" t="s">
-        <v>193</v>
-      </c>
-      <c r="E94" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F94" t="b">
-        <v>1</v>
+        <v>145</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>233</v>
+        <v>193</v>
       </c>
       <c r="B95" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C95" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D95" t="s">
-        <v>213</v>
+        <v>192</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="F95" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B96" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C96" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="D96" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B97" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C97" t="s">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="D97" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B98" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C98" t="s">
-        <v>138</v>
+        <v>4</v>
       </c>
       <c r="D98" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B99" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C99" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D99" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B100" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C100" t="s">
         <v>133</v>
       </c>
       <c r="D100" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B101" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C101" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
       <c r="D101" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B102" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C102" t="s">
         <v>4</v>
       </c>
       <c r="D102" t="s">
-        <v>220</v>
-      </c>
-      <c r="E102" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G102" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B103" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C103" t="s">
-        <v>133</v>
+        <v>4</v>
       </c>
       <c r="D103" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E103" s="7" t="s">
         <v>119</v>
       </c>
       <c r="G103" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B104" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C104" t="s">
-        <v>4</v>
+        <v>133</v>
       </c>
       <c r="D104" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E104" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G104" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>232</v>
+      </c>
+      <c r="B105" t="s">
+        <v>223</v>
+      </c>
+      <c r="C105" t="s">
+        <v>4</v>
+      </c>
+      <c r="D105" t="s">
+        <v>221</v>
+      </c>
+      <c r="E105" s="7" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate to calamine for processing efficiency
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4BC391-9E29-4809-85E3-5D76DBDB0FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02C4135-5F60-4124-AF17-FBAAA4C0A143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="235">
   <si>
     <t>type</t>
   </si>
@@ -459,87 +459,15 @@
     <t>shareholders_funds</t>
   </si>
   <si>
-    <t>Shareholders Funds
-th GBP</t>
-  </si>
-  <si>
-    <t>Profit (Loss) before Taxation
-th GBP</t>
-  </si>
-  <si>
     <t>profit_loss_pretax</t>
   </si>
   <si>
     <t>employees</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of employees
-</t>
-  </si>
-  <si>
     <t>Number of employees</t>
   </si>
   <si>
-    <t>Tangible Assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Land &amp; Buildings
-th GBP</t>
-  </si>
-  <si>
-    <t>Freehold Land
-th GBP</t>
-  </si>
-  <si>
-    <t>Leasehold Land
-th GBP</t>
-  </si>
-  <si>
-    <t>Fixtures &amp; Fittings
-th GBP</t>
-  </si>
-  <si>
-    <t>Plant &amp; Vehicles
-th GBP</t>
-  </si>
-  <si>
-    <t>Plant
-th GBP</t>
-  </si>
-  <si>
-    <t>Vehicles
-th GBP</t>
-  </si>
-  <si>
-    <t>Other Fixed Assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Intangible Assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Investments &amp; other fixed assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Fixed Assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Current Liabilities
-th GBP</t>
-  </si>
-  <si>
-    <t>Total Assets
-th GBP</t>
-  </si>
-  <si>
-    <t>Long Term Liabilities
-th GBP</t>
-  </si>
-  <si>
     <t>a3_assets</t>
   </si>
   <si>
@@ -585,70 +513,6 @@
     <t>fixed_total</t>
   </si>
   <si>
-    <t>Turnover
-th GBP</t>
-  </si>
-  <si>
-    <t>Cost of Sales
-th GBP</t>
-  </si>
-  <si>
-    <t>Administration Expenses
-th GBP</t>
-  </si>
-  <si>
-    <t>Interest Paid
-th GBP</t>
-  </si>
-  <si>
-    <t>Profit (Loss) before Tax
-th GBP</t>
-  </si>
-  <si>
-    <t>Taxation
-th GBP</t>
-  </si>
-  <si>
-    <t>Dividends (Distributable profit)
-th GBP</t>
-  </si>
-  <si>
-    <t>Depreciation
-th GBP</t>
-  </si>
-  <si>
-    <t>Research &amp; Development
-th GBP</t>
-  </si>
-  <si>
-    <t>Remuneration
-th GBP</t>
-  </si>
-  <si>
-    <t>Wages &amp; Salaries
-th GBP</t>
-  </si>
-  <si>
-    <t>Social Security Costs
-th GBP</t>
-  </si>
-  <si>
-    <t>Pension Costs
-th GBP</t>
-  </si>
-  <si>
-    <t>Other Staff Costs
-th GBP</t>
-  </si>
-  <si>
-    <t>Directors' Remuneration
-th GBP</t>
-  </si>
-  <si>
-    <t>EBITDA
-th GBP</t>
-  </si>
-  <si>
     <t>a4_profits</t>
   </si>
   <si>
@@ -715,14 +579,6 @@
     <t>Credit score indicator</t>
   </si>
   <si>
-    <t>Likelihood of failure
-%</t>
-  </si>
-  <si>
-    <t>Credit limit
-GBP</t>
-  </si>
-  <si>
     <t>Previous credit score</t>
   </si>
   <si>
@@ -781,6 +637,108 @@
   </si>
   <si>
     <t>2 special rows that index the below</t>
+  </si>
+  <si>
+    <t>Shareholders Fundsth GBP</t>
+  </si>
+  <si>
+    <t>Profit (Loss) before Taxationth GBP</t>
+  </si>
+  <si>
+    <t>Tangible Assetsth GBP</t>
+  </si>
+  <si>
+    <t>Land &amp; Buildingsth GBP</t>
+  </si>
+  <si>
+    <t>Freehold Landth GBP</t>
+  </si>
+  <si>
+    <t>Leasehold Landth GBP</t>
+  </si>
+  <si>
+    <t>Fixtures &amp; Fittingsth GBP</t>
+  </si>
+  <si>
+    <t>Plant &amp; Vehiclesth GBP</t>
+  </si>
+  <si>
+    <t>Plantth GBP</t>
+  </si>
+  <si>
+    <t>Vehiclesth GBP</t>
+  </si>
+  <si>
+    <t>Other Fixed Assetsth GBP</t>
+  </si>
+  <si>
+    <t>Intangible Assetsth GBP</t>
+  </si>
+  <si>
+    <t>Investments &amp; other fixed assetsth GBP</t>
+  </si>
+  <si>
+    <t>Fixed Assetsth GBP</t>
+  </si>
+  <si>
+    <t>Current Liabilitiesth GBP</t>
+  </si>
+  <si>
+    <t>Total Assetsth GBP</t>
+  </si>
+  <si>
+    <t>Long Term Liabilitiesth GBP</t>
+  </si>
+  <si>
+    <t>Cost of Salesth GBP</t>
+  </si>
+  <si>
+    <t>Administration Expensesth GBP</t>
+  </si>
+  <si>
+    <t>Interest Paidth GBP</t>
+  </si>
+  <si>
+    <t>Profit (Loss) before Taxth GBP</t>
+  </si>
+  <si>
+    <t>Taxationth GBP</t>
+  </si>
+  <si>
+    <t>Dividends (Distributable profit)th GBP</t>
+  </si>
+  <si>
+    <t>Depreciationth GBP</t>
+  </si>
+  <si>
+    <t>Research &amp; Developmentth GBP</t>
+  </si>
+  <si>
+    <t>Remunerationth GBP</t>
+  </si>
+  <si>
+    <t>Wages &amp; Salariesth GBP</t>
+  </si>
+  <si>
+    <t>Social Security Coststh GBP</t>
+  </si>
+  <si>
+    <t>Pension Coststh GBP</t>
+  </si>
+  <si>
+    <t>Other Staff Coststh GBP</t>
+  </si>
+  <si>
+    <t>Directors' Remunerationth GBP</t>
+  </si>
+  <si>
+    <t>EBITDAth GBP</t>
+  </si>
+  <si>
+    <t>Likelihood of failure%</t>
+  </si>
+  <si>
+    <t>Credit limitGBP</t>
   </si>
 </sst>
 </file>
@@ -1283,10 +1241,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1294,6 +1248,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1669,14 +1627,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" customWidth="1"/>
     <col min="3" max="3" width="10.140625" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="7"/>
+    <col min="5" max="5" width="9.140625" style="5"/>
+    <col min="12" max="12" width="43.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1692,7 +1651,7 @@
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="4" t="s">
         <v>104</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1715,7 +1674,7 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F2" t="b">
@@ -1738,7 +1697,7 @@
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>118</v>
       </c>
       <c r="F3" t="b">
@@ -1758,7 +1717,7 @@
       <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>119</v>
       </c>
       <c r="G4" t="s">
@@ -2033,7 +1992,7 @@
       <c r="D23" t="s">
         <v>42</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F23" t="b">
@@ -2056,7 +2015,7 @@
       <c r="D24" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F24" t="b">
@@ -2076,7 +2035,7 @@
       <c r="D25" t="s">
         <v>46</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F25" t="b">
@@ -2113,7 +2072,7 @@
       <c r="D27" t="s">
         <v>50</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E27" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F27" t="b">
@@ -2150,7 +2109,7 @@
       <c r="D29" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E29" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F29" t="b">
@@ -2173,7 +2132,7 @@
       <c r="D30" t="s">
         <v>56</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E30" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F30" t="b">
@@ -2207,13 +2166,13 @@
       <c r="D32" t="s">
         <v>60</v>
       </c>
-      <c r="E32" s="7" t="b">
+      <c r="E32" s="5" t="b">
         <v>0</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="7" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2230,7 +2189,7 @@
       <c r="D33" t="s">
         <v>62</v>
       </c>
-      <c r="H33" s="4"/>
+      <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -2245,7 +2204,7 @@
       <c r="D34" t="s">
         <v>64</v>
       </c>
-      <c r="H34" s="4"/>
+      <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -2260,7 +2219,7 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-      <c r="H35" s="4"/>
+      <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
@@ -2275,7 +2234,7 @@
       <c r="D36" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="4"/>
+      <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -2290,7 +2249,7 @@
       <c r="D37" t="s">
         <v>70</v>
       </c>
-      <c r="H37" s="4"/>
+      <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
@@ -2305,7 +2264,7 @@
       <c r="D38" t="s">
         <v>72</v>
       </c>
-      <c r="H38" s="4"/>
+      <c r="H38" s="7"/>
     </row>
     <row r="39" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -2320,7 +2279,7 @@
       <c r="D39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H39" s="4"/>
+      <c r="H39" s="7"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -2335,7 +2294,7 @@
       <c r="D40" t="s">
         <v>75</v>
       </c>
-      <c r="H40" s="4"/>
+      <c r="H40" s="7"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -2350,7 +2309,7 @@
       <c r="D41" t="s">
         <v>77</v>
       </c>
-      <c r="H41" s="4"/>
+      <c r="H41" s="7"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
@@ -2365,7 +2324,7 @@
       <c r="D42" t="s">
         <v>79</v>
       </c>
-      <c r="H42" s="4"/>
+      <c r="H42" s="7"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
@@ -2380,7 +2339,7 @@
       <c r="D43" t="s">
         <v>81</v>
       </c>
-      <c r="H43" s="4"/>
+      <c r="H43" s="7"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
@@ -2395,7 +2354,7 @@
       <c r="D44" t="s">
         <v>83</v>
       </c>
-      <c r="H44" s="4"/>
+      <c r="H44" s="7"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -2410,7 +2369,7 @@
       <c r="D45" t="s">
         <v>85</v>
       </c>
-      <c r="H45" s="4"/>
+      <c r="H45" s="7"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
@@ -2425,7 +2384,7 @@
       <c r="D46" t="s">
         <v>87</v>
       </c>
-      <c r="H46" s="4"/>
+      <c r="H46" s="7"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
@@ -2440,7 +2399,7 @@
       <c r="D47" t="s">
         <v>89</v>
       </c>
-      <c r="H47" s="4"/>
+      <c r="H47" s="7"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
@@ -2455,9 +2414,9 @@
       <c r="D48" t="s">
         <v>91</v>
       </c>
-      <c r="H48" s="4"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48" s="7"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -2470,14 +2429,14 @@
       <c r="D49" t="s">
         <v>94</v>
       </c>
-      <c r="E49" s="7" t="s">
+      <c r="E49" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F49" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -2490,104 +2449,104 @@
       <c r="D50" t="s">
         <v>96</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="E50" s="5" t="s">
         <v>119</v>
       </c>
       <c r="F50" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>123</v>
       </c>
       <c r="C51" t="s">
         <v>97</v>
       </c>
-      <c r="E51" s="7" t="s">
+      <c r="E51" s="5" t="s">
         <v>117</v>
       </c>
       <c r="G51" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>124</v>
       </c>
       <c r="C52" t="s">
         <v>97</v>
       </c>
-      <c r="E52" s="7" t="s">
+      <c r="E52" s="5" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>107</v>
       </c>
       <c r="C53" t="s">
         <v>97</v>
       </c>
-      <c r="E53" s="7" t="s">
+      <c r="E53" s="5" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>131</v>
       </c>
       <c r="C54" t="s">
         <v>97</v>
       </c>
-      <c r="E54" s="7" t="s">
+      <c r="E54" s="5" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>129</v>
       </c>
       <c r="C55" t="s">
         <v>127</v>
       </c>
-      <c r="E55" s="7" t="s">
+      <c r="E55" s="5" t="s">
         <v>117</v>
       </c>
       <c r="G55" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>126</v>
       </c>
       <c r="C56" t="s">
         <v>127</v>
       </c>
-      <c r="E56" s="7" t="s">
+      <c r="E56" s="5" t="s">
         <v>117</v>
       </c>
       <c r="G56" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="8" t="s">
-        <v>235</v>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B57" s="6" t="s">
+        <v>199</v>
       </c>
       <c r="C57" t="s">
         <v>127</v>
       </c>
-      <c r="E57" s="7" t="s">
+      <c r="E57" s="5" t="s">
         <v>120</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B58" s="6" t="s">
         <v>121</v>
       </c>
       <c r="C58" t="s">
@@ -2596,14 +2555,14 @@
       <c r="D58" t="s">
         <v>122</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="E58" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F58" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>134</v>
       </c>
@@ -2613,14 +2572,14 @@
       <c r="C59" t="s">
         <v>97</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="D59" t="s">
         <v>136</v>
       </c>
-      <c r="E59" s="7" t="s">
+      <c r="E59" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>134</v>
       </c>
@@ -2630,17 +2589,18 @@
       <c r="C60" t="s">
         <v>138</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" t="s">
         <v>139</v>
       </c>
-      <c r="E60" s="7" t="s">
+      <c r="E60" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F60" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L60" s="8"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>134</v>
       </c>
@@ -2650,751 +2610,796 @@
       <c r="C61" t="s">
         <v>138</v>
       </c>
-      <c r="D61" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="E61" s="7" t="s">
+      <c r="D61" t="s">
+        <v>201</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F61" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L61" s="8"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C62" t="s">
         <v>138</v>
       </c>
-      <c r="D62" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E62" s="7" t="s">
+      <c r="D62" t="s">
+        <v>202</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F62" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L62" s="8"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>134</v>
       </c>
       <c r="B63" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C63" t="s">
         <v>133</v>
       </c>
-      <c r="D63" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E63" s="7" t="s">
+      <c r="D63" t="s">
+        <v>143</v>
+      </c>
+      <c r="E63" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F63" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L63" s="8"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B64" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="C64" t="s">
         <v>138</v>
       </c>
-      <c r="D64" t="s">
-        <v>147</v>
-      </c>
-      <c r="E64" s="7" t="s">
+      <c r="D64" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E64" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F64" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L64" s="8"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B65" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="C65" t="s">
         <v>138</v>
       </c>
       <c r="D65" t="s">
+        <v>204</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L65" s="8"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>144</v>
+      </c>
+      <c r="B66" t="s">
         <v>148</v>
       </c>
-      <c r="E65" s="7" t="s">
+      <c r="C66" t="s">
+        <v>138</v>
+      </c>
+      <c r="D66" t="s">
+        <v>205</v>
+      </c>
+      <c r="E66" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>162</v>
-      </c>
-      <c r="B66" t="s">
-        <v>166</v>
-      </c>
-      <c r="C66" t="s">
-        <v>138</v>
-      </c>
-      <c r="D66" t="s">
+      <c r="L66" s="8"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>144</v>
+      </c>
+      <c r="B67" t="s">
         <v>149</v>
       </c>
-      <c r="E66" s="7" t="s">
+      <c r="C67" t="s">
+        <v>138</v>
+      </c>
+      <c r="D67" t="s">
+        <v>206</v>
+      </c>
+      <c r="E67" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>162</v>
-      </c>
-      <c r="B67" t="s">
-        <v>167</v>
-      </c>
-      <c r="C67" t="s">
-        <v>138</v>
-      </c>
-      <c r="D67" t="s">
+      <c r="L67" s="8"/>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>144</v>
+      </c>
+      <c r="B68" t="s">
+        <v>160</v>
+      </c>
+      <c r="C68" t="s">
+        <v>138</v>
+      </c>
+      <c r="D68" t="s">
+        <v>207</v>
+      </c>
+      <c r="L68" s="8"/>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>144</v>
+      </c>
+      <c r="B69" t="s">
         <v>150</v>
       </c>
-      <c r="E67" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>162</v>
-      </c>
-      <c r="B68" t="s">
-        <v>194</v>
-      </c>
-      <c r="C68" t="s">
-        <v>138</v>
-      </c>
-      <c r="D68" t="s">
+      <c r="C69" t="s">
+        <v>138</v>
+      </c>
+      <c r="D69" t="s">
+        <v>208</v>
+      </c>
+      <c r="L69" s="8"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>144</v>
+      </c>
+      <c r="B70" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>162</v>
-      </c>
-      <c r="B69" t="s">
-        <v>168</v>
-      </c>
-      <c r="C69" t="s">
-        <v>138</v>
-      </c>
-      <c r="D69" t="s">
+      <c r="C70" t="s">
+        <v>138</v>
+      </c>
+      <c r="D70" t="s">
+        <v>209</v>
+      </c>
+      <c r="L70" s="8"/>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>144</v>
+      </c>
+      <c r="B71" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>162</v>
-      </c>
-      <c r="B70" t="s">
-        <v>169</v>
-      </c>
-      <c r="C70" t="s">
-        <v>138</v>
-      </c>
-      <c r="D70" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>162</v>
-      </c>
-      <c r="B71" t="s">
-        <v>170</v>
-      </c>
       <c r="C71" t="s">
         <v>138</v>
       </c>
       <c r="D71" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+      <c r="L71" s="8"/>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B72" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="C72" t="s">
         <v>138</v>
       </c>
       <c r="D72" t="s">
-        <v>155</v>
-      </c>
-      <c r="E72" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="E72" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F72" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L72" s="8"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B73" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="C73" t="s">
         <v>138</v>
       </c>
       <c r="D73" t="s">
-        <v>156</v>
-      </c>
-      <c r="E73" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="E73" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F73" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L73" s="8"/>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B74" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="C74" t="s">
         <v>138</v>
       </c>
       <c r="D74" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+      <c r="L74" s="8"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B75" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="C75" t="s">
         <v>138</v>
       </c>
       <c r="D75" t="s">
-        <v>158</v>
-      </c>
-      <c r="E75" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L75" s="8"/>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B76" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="C76" t="s">
         <v>138</v>
       </c>
       <c r="D76" t="s">
-        <v>159</v>
-      </c>
-      <c r="E76" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L76" s="8"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B77" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="C77" t="s">
         <v>138</v>
       </c>
       <c r="D77" t="s">
-        <v>160</v>
-      </c>
-      <c r="E77" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F77" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L77" s="8"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B78" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="C78" t="s">
         <v>138</v>
       </c>
       <c r="D78" t="s">
-        <v>161</v>
-      </c>
-      <c r="E78" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F78" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L78" s="8"/>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B79" t="s">
-        <v>199</v>
+        <v>165</v>
       </c>
       <c r="C79" t="s">
         <v>138</v>
       </c>
       <c r="D79" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="L79" s="8"/>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>161</v>
       </c>
       <c r="C80" t="s">
         <v>138</v>
       </c>
       <c r="D80" t="s">
-        <v>178</v>
-      </c>
-      <c r="E80" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E80" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F80" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L80" s="8"/>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B81" t="s">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="C81" t="s">
         <v>138</v>
       </c>
       <c r="D81" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+      <c r="L81" s="8"/>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B82" t="s">
-        <v>198</v>
+        <v>164</v>
       </c>
       <c r="C82" t="s">
         <v>138</v>
       </c>
       <c r="D82" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="L82" s="8"/>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B83" t="s">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="C83" t="s">
         <v>138</v>
       </c>
       <c r="D83" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+      <c r="L83" s="8"/>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B84" t="s">
-        <v>196</v>
+        <v>162</v>
       </c>
       <c r="C84" t="s">
         <v>138</v>
       </c>
       <c r="D84" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+      <c r="L84" s="8"/>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B85" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="C85" t="s">
         <v>138</v>
       </c>
       <c r="D85" t="s">
-        <v>183</v>
-      </c>
-      <c r="E85" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F85" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L85" s="8"/>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B86" t="s">
-        <v>202</v>
+        <v>168</v>
       </c>
       <c r="C86" t="s">
         <v>138</v>
       </c>
       <c r="D86" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+      <c r="L86" s="8"/>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B87" t="s">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="C87" t="s">
         <v>138</v>
       </c>
       <c r="D87" t="s">
-        <v>185</v>
-      </c>
-      <c r="E87" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="E87" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F87" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L87" s="8"/>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B88" t="s">
-        <v>209</v>
+        <v>175</v>
       </c>
       <c r="C88" t="s">
         <v>138</v>
       </c>
       <c r="D88" t="s">
-        <v>186</v>
-      </c>
-      <c r="E88" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L88" s="8"/>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B89" t="s">
-        <v>204</v>
+        <v>170</v>
       </c>
       <c r="C89" t="s">
         <v>138</v>
       </c>
       <c r="D89" t="s">
-        <v>187</v>
-      </c>
-      <c r="E89" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F89" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L89" s="8"/>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B90" t="s">
-        <v>205</v>
+        <v>171</v>
       </c>
       <c r="C90" t="s">
         <v>138</v>
       </c>
       <c r="D90" t="s">
-        <v>188</v>
-      </c>
-      <c r="E90" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E90" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F90" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L90" s="8"/>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B91" t="s">
-        <v>206</v>
+        <v>172</v>
       </c>
       <c r="C91" t="s">
         <v>138</v>
       </c>
       <c r="D91" t="s">
-        <v>189</v>
-      </c>
-      <c r="E91" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="E91" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F91" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L91" s="8"/>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B92" t="s">
-        <v>207</v>
+        <v>173</v>
       </c>
       <c r="C92" t="s">
         <v>138</v>
       </c>
       <c r="D92" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+      <c r="L92" s="8"/>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B93" t="s">
-        <v>208</v>
+        <v>174</v>
       </c>
       <c r="C93" t="s">
         <v>138</v>
       </c>
       <c r="D93" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+      <c r="L93" s="8"/>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B94" t="s">
-        <v>210</v>
+        <v>176</v>
       </c>
       <c r="C94" t="s">
         <v>138</v>
       </c>
       <c r="D94" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+      <c r="L94" s="8"/>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>193</v>
+        <v>159</v>
       </c>
       <c r="B95" t="s">
-        <v>211</v>
+        <v>177</v>
       </c>
       <c r="C95" t="s">
         <v>138</v>
       </c>
       <c r="D95" t="s">
-        <v>192</v>
-      </c>
-      <c r="E95" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="E95" s="5" t="s">
         <v>120</v>
       </c>
       <c r="F95" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="L95" s="8"/>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B96" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="C96" t="s">
         <v>133</v>
       </c>
       <c r="D96" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+        <v>178</v>
+      </c>
+      <c r="L96" s="8"/>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B97" t="s">
-        <v>224</v>
+        <v>188</v>
       </c>
       <c r="C97" t="s">
         <v>93</v>
       </c>
       <c r="D97" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+      <c r="L97" s="8"/>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B98" t="s">
-        <v>225</v>
+        <v>189</v>
       </c>
       <c r="C98" t="s">
         <v>4</v>
       </c>
       <c r="D98" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+      <c r="L98" s="8"/>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B99" t="s">
-        <v>226</v>
+        <v>190</v>
       </c>
       <c r="C99" t="s">
         <v>138</v>
       </c>
       <c r="D99" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+      <c r="L99" s="8"/>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B100" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="C100" t="s">
         <v>133</v>
       </c>
       <c r="D100" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+      <c r="L100" s="8"/>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B101" t="s">
-        <v>228</v>
+        <v>192</v>
       </c>
       <c r="C101" t="s">
         <v>133</v>
       </c>
       <c r="D101" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+      <c r="L101" s="8"/>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B102" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="C102" t="s">
         <v>4</v>
       </c>
       <c r="D102" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+      <c r="L102" s="8"/>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B103" t="s">
-        <v>230</v>
+        <v>194</v>
       </c>
       <c r="C103" t="s">
         <v>4</v>
       </c>
       <c r="D103" t="s">
-        <v>219</v>
-      </c>
-      <c r="E103" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E103" s="5" t="s">
         <v>119</v>
       </c>
       <c r="G103" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+      <c r="L103" s="8"/>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B104" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="C104" t="s">
         <v>133</v>
       </c>
       <c r="D104" t="s">
-        <v>220</v>
-      </c>
-      <c r="E104" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="E104" s="5" t="s">
         <v>119</v>
       </c>
       <c r="G104" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+      <c r="L104" s="8"/>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="B105" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="C105" t="s">
         <v>4</v>
       </c>
       <c r="D105" t="s">
-        <v>221</v>
-      </c>
-      <c r="E105" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="E105" s="5" t="s">
         <v>119</v>
       </c>
+      <c r="L105" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Handled duplication and efficiency
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02C4135-5F60-4124-AF17-FBAAA4C0A143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C928DE-1A45-415A-912F-AFB0D5895F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="237">
   <si>
     <t>type</t>
   </si>
@@ -414,18 +414,9 @@
 Strategy, organization and policy</t>
   </si>
   <si>
-    <t>file_code</t>
-  </si>
-  <si>
     <t>str</t>
   </si>
   <si>
-    <t>From the filepaths</t>
-  </si>
-  <si>
-    <t>industry_code</t>
-  </si>
-  <si>
     <t>same as company_name for most, missing for others. Lars calls it 'company_name_B</t>
   </si>
   <si>
@@ -739,6 +730,21 @@
   </si>
   <si>
     <t>Credit limitGBP</t>
+  </si>
+  <si>
+    <t>may_mix</t>
+  </si>
+  <si>
+    <t>industry_codes</t>
+  </si>
+  <si>
+    <t>file_codes</t>
+  </si>
+  <si>
+    <t>When there are duplicates, store them here comma separated</t>
+  </si>
+  <si>
+    <t>We will need to parse these a list</t>
   </si>
 </sst>
 </file>
@@ -1234,7 +1240,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1251,7 +1257,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1627,7 +1632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1635,10 +1640,10 @@
     <col min="3" max="3" width="10.140625" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="9.140625" style="5"/>
-    <col min="12" max="12" width="43.85546875" customWidth="1"/>
+    <col min="13" max="13" width="43.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
@@ -1658,10 +1663,13 @@
         <v>111</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1680,11 +1688,11 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>118</v>
       </c>
@@ -1703,8 +1711,11 @@
       <c r="F3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1720,11 +1731,11 @@
       <c r="E4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1737,11 +1748,11 @@
       <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1755,7 +1766,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1769,7 +1780,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1783,7 +1794,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1797,7 +1808,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1811,7 +1822,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1825,7 +1836,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1839,7 +1850,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1853,7 +1864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -1867,7 +1878,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -1881,7 +1892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1895,7 +1906,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1909,7 +1920,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -1923,7 +1934,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -1937,7 +1948,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -1951,7 +1962,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>2</v>
       </c>
@@ -1965,7 +1976,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -1979,7 +1990,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -1998,11 +2009,11 @@
       <c r="F23" t="b">
         <v>0</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -2022,7 +2033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -2042,7 +2053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -2050,16 +2061,19 @@
         <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D26" t="s">
         <v>48</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -2078,11 +2092,11 @@
       <c r="F27" t="b">
         <v>1</v>
       </c>
-      <c r="G27" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -2096,7 +2110,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -2104,7 +2118,7 @@
         <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D29" t="s">
         <v>54</v>
@@ -2115,11 +2129,11 @@
       <c r="F29" t="b">
         <v>1</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -2139,7 +2153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -2153,7 +2167,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -2166,17 +2180,14 @@
       <c r="D32" t="s">
         <v>60</v>
       </c>
-      <c r="E32" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="2" t="s">
+      <c r="H32" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="I32" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -2189,9 +2200,9 @@
       <c r="D33" t="s">
         <v>62</v>
       </c>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I33" s="7"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -2204,9 +2215,9 @@
       <c r="D34" t="s">
         <v>64</v>
       </c>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I34" s="7"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -2219,9 +2230,9 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-      <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I35" s="7"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>2</v>
       </c>
@@ -2234,9 +2245,9 @@
       <c r="D36" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="7"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I36" s="7"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -2249,9 +2260,9 @@
       <c r="D37" t="s">
         <v>70</v>
       </c>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I37" s="7"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -2264,9 +2275,9 @@
       <c r="D38" t="s">
         <v>72</v>
       </c>
-      <c r="H38" s="7"/>
-    </row>
-    <row r="39" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I38" s="7"/>
+    </row>
+    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -2279,9 +2290,9 @@
       <c r="D39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H39" s="7"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I39" s="7"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -2294,9 +2305,9 @@
       <c r="D40" t="s">
         <v>75</v>
       </c>
-      <c r="H40" s="7"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I40" s="7"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -2309,9 +2320,9 @@
       <c r="D41" t="s">
         <v>77</v>
       </c>
-      <c r="H41" s="7"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I41" s="7"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -2324,9 +2335,9 @@
       <c r="D42" t="s">
         <v>79</v>
       </c>
-      <c r="H42" s="7"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I42" s="7"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>2</v>
       </c>
@@ -2339,9 +2350,9 @@
       <c r="D43" t="s">
         <v>81</v>
       </c>
-      <c r="H43" s="7"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I43" s="7"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -2354,9 +2365,9 @@
       <c r="D44" t="s">
         <v>83</v>
       </c>
-      <c r="H44" s="7"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I44" s="7"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>2</v>
       </c>
@@ -2369,9 +2380,9 @@
       <c r="D45" t="s">
         <v>85</v>
       </c>
-      <c r="H45" s="7"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I45" s="7"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -2384,9 +2395,9 @@
       <c r="D46" t="s">
         <v>87</v>
       </c>
-      <c r="H46" s="7"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I46" s="7"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -2399,9 +2410,9 @@
       <c r="D47" t="s">
         <v>89</v>
       </c>
-      <c r="H47" s="7"/>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I47" s="7"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2414,9 +2425,9 @@
       <c r="D48" t="s">
         <v>91</v>
       </c>
-      <c r="H48" s="7"/>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I48" s="7"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -2436,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -2444,7 +2455,7 @@
         <v>95</v>
       </c>
       <c r="C50" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D50" t="s">
         <v>96</v>
@@ -2455,8 +2466,11 @@
       <c r="F50" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>123</v>
       </c>
@@ -2466,11 +2480,11 @@
       <c r="E51" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G51" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H51" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>124</v>
       </c>
@@ -2481,7 +2495,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>107</v>
       </c>
@@ -2492,9 +2506,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C54" t="s">
         <v>97</v>
@@ -2503,54 +2517,60 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>118</v>
+      </c>
       <c r="B55" t="s">
-        <v>129</v>
+        <v>233</v>
       </c>
       <c r="C55" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G55" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H55" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>118</v>
+      </c>
       <c r="B56" t="s">
+        <v>234</v>
+      </c>
+      <c r="C56" t="s">
         <v>126</v>
-      </c>
-      <c r="C56" t="s">
-        <v>127</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G56" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H56" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B57" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C57" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H57" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B58" s="6" t="s">
         <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D58" t="s">
         <v>122</v>
@@ -2562,35 +2582,35 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B59" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C59" t="s">
         <v>97</v>
       </c>
       <c r="D59" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E59" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>131</v>
+      </c>
+      <c r="B60" t="s">
         <v>134</v>
       </c>
-      <c r="B60" t="s">
-        <v>137</v>
-      </c>
       <c r="C60" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D60" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>120</v>
@@ -2598,20 +2618,19 @@
       <c r="F60" t="b">
         <v>1</v>
       </c>
-      <c r="L60" s="8"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C61" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D61" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>120</v>
@@ -2619,20 +2638,19 @@
       <c r="F61" t="b">
         <v>1</v>
       </c>
-      <c r="L61" s="8"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B62" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C62" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D62" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>120</v>
@@ -2640,20 +2658,19 @@
       <c r="F62" t="b">
         <v>1</v>
       </c>
-      <c r="L62" s="8"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B63" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C63" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D63" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>120</v>
@@ -2661,20 +2678,19 @@
       <c r="F63" t="b">
         <v>1</v>
       </c>
-      <c r="L63" s="8"/>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B64" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C64" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>120</v>
@@ -2682,134 +2698,126 @@
       <c r="F64" t="b">
         <v>1</v>
       </c>
-      <c r="L64" s="8"/>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>141</v>
+      </c>
+      <c r="B65" t="s">
         <v>144</v>
       </c>
-      <c r="B65" t="s">
-        <v>147</v>
-      </c>
       <c r="C65" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D65" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L65" s="8"/>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B66" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C66" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D66" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E66" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L66" s="8"/>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B67" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C67" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D67" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E67" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L67" s="8"/>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B68" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C68" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D68" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>141</v>
+      </c>
+      <c r="B69" t="s">
+        <v>147</v>
+      </c>
+      <c r="C69" t="s">
+        <v>135</v>
+      </c>
+      <c r="D69" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>141</v>
+      </c>
+      <c r="B70" t="s">
+        <v>148</v>
+      </c>
+      <c r="C70" t="s">
+        <v>135</v>
+      </c>
+      <c r="D70" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>141</v>
+      </c>
+      <c r="B71" t="s">
+        <v>149</v>
+      </c>
+      <c r="C71" t="s">
+        <v>135</v>
+      </c>
+      <c r="D71" t="s">
         <v>207</v>
       </c>
-      <c r="L68" s="8"/>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>144</v>
-      </c>
-      <c r="B69" t="s">
-        <v>150</v>
-      </c>
-      <c r="C69" t="s">
-        <v>138</v>
-      </c>
-      <c r="D69" t="s">
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>141</v>
+      </c>
+      <c r="B72" t="s">
+        <v>154</v>
+      </c>
+      <c r="C72" t="s">
+        <v>135</v>
+      </c>
+      <c r="D72" t="s">
         <v>208</v>
-      </c>
-      <c r="L69" s="8"/>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>144</v>
-      </c>
-      <c r="B70" t="s">
-        <v>151</v>
-      </c>
-      <c r="C70" t="s">
-        <v>138</v>
-      </c>
-      <c r="D70" t="s">
-        <v>209</v>
-      </c>
-      <c r="L70" s="8"/>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>144</v>
-      </c>
-      <c r="B71" t="s">
-        <v>152</v>
-      </c>
-      <c r="C71" t="s">
-        <v>138</v>
-      </c>
-      <c r="D71" t="s">
-        <v>210</v>
-      </c>
-      <c r="L71" s="8"/>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>144</v>
-      </c>
-      <c r="B72" t="s">
-        <v>157</v>
-      </c>
-      <c r="C72" t="s">
-        <v>138</v>
-      </c>
-      <c r="D72" t="s">
-        <v>211</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>120</v>
@@ -2817,20 +2825,19 @@
       <c r="F72" t="b">
         <v>1</v>
       </c>
-      <c r="L72" s="8"/>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B73" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C73" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D73" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>120</v>
@@ -2838,35 +2845,33 @@
       <c r="F73" t="b">
         <v>1</v>
       </c>
-      <c r="L73" s="8"/>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B74" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C74" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D74" t="s">
-        <v>213</v>
-      </c>
-      <c r="L74" s="8"/>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B75" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C75" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D75" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>120</v>
@@ -2874,38 +2879,36 @@
       <c r="F75" t="b">
         <v>1</v>
       </c>
-      <c r="L75" s="8"/>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B76" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C76" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D76" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L76" s="8"/>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C77" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D77" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>120</v>
@@ -2913,20 +2916,19 @@
       <c r="F77" t="b">
         <v>1</v>
       </c>
-      <c r="L77" s="8"/>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C78" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D78" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E78" s="5" t="s">
         <v>120</v>
@@ -2934,35 +2936,33 @@
       <c r="F78" t="b">
         <v>1</v>
       </c>
-      <c r="L78" s="8"/>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B79" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C79" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D79" t="s">
-        <v>139</v>
-      </c>
-      <c r="L79" s="8"/>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B80" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C80" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D80" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>120</v>
@@ -2970,80 +2970,75 @@
       <c r="F80" t="b">
         <v>1</v>
       </c>
-      <c r="L80" s="8"/>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>156</v>
+      </c>
+      <c r="B81" t="s">
+        <v>160</v>
+      </c>
+      <c r="C81" t="s">
+        <v>135</v>
+      </c>
+      <c r="D81" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>156</v>
+      </c>
+      <c r="B82" t="s">
+        <v>161</v>
+      </c>
+      <c r="C82" t="s">
+        <v>135</v>
+      </c>
+      <c r="D82" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>156</v>
+      </c>
+      <c r="B83" t="s">
+        <v>163</v>
+      </c>
+      <c r="C83" t="s">
+        <v>135</v>
+      </c>
+      <c r="D83" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>156</v>
+      </c>
+      <c r="B84" t="s">
         <v>159</v>
       </c>
-      <c r="B81" t="s">
-        <v>163</v>
-      </c>
-      <c r="C81" t="s">
-        <v>138</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="C84" t="s">
+        <v>135</v>
+      </c>
+      <c r="D84" t="s">
         <v>219</v>
       </c>
-      <c r="L81" s="8"/>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>159</v>
-      </c>
-      <c r="B82" t="s">
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>156</v>
+      </c>
+      <c r="B85" t="s">
         <v>164</v>
       </c>
-      <c r="C82" t="s">
-        <v>138</v>
-      </c>
-      <c r="D82" t="s">
+      <c r="C85" t="s">
+        <v>135</v>
+      </c>
+      <c r="D85" t="s">
         <v>220</v>
-      </c>
-      <c r="L82" s="8"/>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>159</v>
-      </c>
-      <c r="B83" t="s">
-        <v>166</v>
-      </c>
-      <c r="C83" t="s">
-        <v>138</v>
-      </c>
-      <c r="D83" t="s">
-        <v>221</v>
-      </c>
-      <c r="L83" s="8"/>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>159</v>
-      </c>
-      <c r="B84" t="s">
-        <v>162</v>
-      </c>
-      <c r="C84" t="s">
-        <v>138</v>
-      </c>
-      <c r="D84" t="s">
-        <v>222</v>
-      </c>
-      <c r="L84" s="8"/>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>159</v>
-      </c>
-      <c r="B85" t="s">
-        <v>167</v>
-      </c>
-      <c r="C85" t="s">
-        <v>138</v>
-      </c>
-      <c r="D85" t="s">
-        <v>223</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>120</v>
@@ -3051,35 +3046,33 @@
       <c r="F85" t="b">
         <v>1</v>
       </c>
-      <c r="L85" s="8"/>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B86" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C86" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D86" t="s">
-        <v>224</v>
-      </c>
-      <c r="L86" s="8"/>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C87" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D87" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>120</v>
@@ -3087,38 +3080,36 @@
       <c r="F87" t="b">
         <v>1</v>
       </c>
-      <c r="L87" s="8"/>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B88" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C88" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D88" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="L88" s="8"/>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B89" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C89" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D89" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>120</v>
@@ -3126,20 +3117,19 @@
       <c r="F89" t="b">
         <v>1</v>
       </c>
-      <c r="L89" s="8"/>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B90" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C90" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D90" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>120</v>
@@ -3147,20 +3137,19 @@
       <c r="F90" t="b">
         <v>1</v>
       </c>
-      <c r="L90" s="8"/>
-    </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B91" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C91" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D91" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>120</v>
@@ -3168,65 +3157,61 @@
       <c r="F91" t="b">
         <v>1</v>
       </c>
-      <c r="L91" s="8"/>
-    </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B92" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" t="s">
+        <v>135</v>
+      </c>
+      <c r="D92" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>156</v>
+      </c>
+      <c r="B93" t="s">
+        <v>171</v>
+      </c>
+      <c r="C93" t="s">
+        <v>135</v>
+      </c>
+      <c r="D93" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>156</v>
+      </c>
+      <c r="B94" t="s">
         <v>173</v>
       </c>
-      <c r="C92" t="s">
-        <v>138</v>
-      </c>
-      <c r="D92" t="s">
-        <v>230</v>
-      </c>
-      <c r="L92" s="8"/>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>159</v>
-      </c>
-      <c r="B93" t="s">
+      <c r="C94" t="s">
+        <v>135</v>
+      </c>
+      <c r="D94" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>156</v>
+      </c>
+      <c r="B95" t="s">
         <v>174</v>
       </c>
-      <c r="C93" t="s">
-        <v>138</v>
-      </c>
-      <c r="D93" t="s">
-        <v>231</v>
-      </c>
-      <c r="L93" s="8"/>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>159</v>
-      </c>
-      <c r="B94" t="s">
-        <v>176</v>
-      </c>
-      <c r="C94" t="s">
-        <v>138</v>
-      </c>
-      <c r="D94" t="s">
-        <v>143</v>
-      </c>
-      <c r="L94" s="8"/>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>159</v>
-      </c>
-      <c r="B95" t="s">
-        <v>177</v>
-      </c>
       <c r="C95" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D95" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>120</v>
@@ -3234,176 +3219,177 @@
       <c r="F95" t="b">
         <v>1</v>
       </c>
-      <c r="L95" s="8"/>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B96" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C96" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D96" t="s">
-        <v>178</v>
-      </c>
-      <c r="L96" s="8"/>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+      <c r="G96" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B97" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C97" t="s">
         <v>93</v>
       </c>
       <c r="D97" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>193</v>
+      </c>
+      <c r="B98" t="s">
+        <v>186</v>
+      </c>
+      <c r="C98" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>193</v>
+      </c>
+      <c r="B99" t="s">
+        <v>187</v>
+      </c>
+      <c r="C99" t="s">
+        <v>135</v>
+      </c>
+      <c r="D99" t="s">
+        <v>230</v>
+      </c>
+      <c r="G99" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>193</v>
+      </c>
+      <c r="B100" t="s">
+        <v>188</v>
+      </c>
+      <c r="C100" t="s">
+        <v>130</v>
+      </c>
+      <c r="D100" t="s">
+        <v>231</v>
+      </c>
+      <c r="G100" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>193</v>
+      </c>
+      <c r="B101" t="s">
+        <v>189</v>
+      </c>
+      <c r="C101" t="s">
+        <v>130</v>
+      </c>
+      <c r="D101" t="s">
+        <v>178</v>
+      </c>
+      <c r="G101" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>193</v>
+      </c>
+      <c r="B102" t="s">
+        <v>190</v>
+      </c>
+      <c r="C102" t="s">
+        <v>4</v>
+      </c>
+      <c r="D102" t="s">
         <v>179</v>
       </c>
-      <c r="L97" s="8"/>
-    </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>196</v>
-      </c>
-      <c r="B98" t="s">
-        <v>189</v>
-      </c>
-      <c r="C98" t="s">
-        <v>4</v>
-      </c>
-      <c r="D98" t="s">
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>193</v>
+      </c>
+      <c r="B103" t="s">
+        <v>191</v>
+      </c>
+      <c r="C103" t="s">
+        <v>4</v>
+      </c>
+      <c r="D103" t="s">
         <v>180</v>
-      </c>
-      <c r="L98" s="8"/>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>196</v>
-      </c>
-      <c r="B99" t="s">
-        <v>190</v>
-      </c>
-      <c r="C99" t="s">
-        <v>138</v>
-      </c>
-      <c r="D99" t="s">
-        <v>233</v>
-      </c>
-      <c r="L99" s="8"/>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>196</v>
-      </c>
-      <c r="B100" t="s">
-        <v>191</v>
-      </c>
-      <c r="C100" t="s">
-        <v>133</v>
-      </c>
-      <c r="D100" t="s">
-        <v>234</v>
-      </c>
-      <c r="L100" s="8"/>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>196</v>
-      </c>
-      <c r="B101" t="s">
-        <v>192</v>
-      </c>
-      <c r="C101" t="s">
-        <v>133</v>
-      </c>
-      <c r="D101" t="s">
-        <v>181</v>
-      </c>
-      <c r="L101" s="8"/>
-    </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>196</v>
-      </c>
-      <c r="B102" t="s">
-        <v>193</v>
-      </c>
-      <c r="C102" t="s">
-        <v>4</v>
-      </c>
-      <c r="D102" t="s">
-        <v>182</v>
-      </c>
-      <c r="L102" s="8"/>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>196</v>
-      </c>
-      <c r="B103" t="s">
-        <v>194</v>
-      </c>
-      <c r="C103" t="s">
-        <v>4</v>
-      </c>
-      <c r="D103" t="s">
-        <v>183</v>
       </c>
       <c r="E103" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G103" t="s">
-        <v>197</v>
-      </c>
-      <c r="L103" s="8"/>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H103" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B104" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C104" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D104" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G104" t="s">
-        <v>198</v>
-      </c>
-      <c r="L104" s="8"/>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H104" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B105" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C105" t="s">
         <v>4</v>
       </c>
       <c r="D105" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="L105" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="H32:H48"/>
+    <mergeCell ref="I32:I48"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Installed yearly_data handling and imported Lars data. pre-first run
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C928DE-1A45-415A-912F-AFB0D5895F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0348AC0-FD8C-4A53-AB52-84701DE9209E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="235">
   <si>
     <t>type</t>
   </si>
@@ -622,12 +622,6 @@
   </si>
   <si>
     <t>number of other firms in the same group</t>
-  </si>
-  <si>
-    <t>fame_key</t>
-  </si>
-  <si>
-    <t>2 special rows that index the below</t>
   </si>
   <si>
     <t>Shareholders Fundsth GBP</t>
@@ -1632,7 +1626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1663,7 +1657,7 @@
         <v>111</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>105</v>
@@ -1748,6 +1742,9 @@
       <c r="D5" t="s">
         <v>11</v>
       </c>
+      <c r="E5" s="5" t="s">
+        <v>119</v>
+      </c>
       <c r="I5" t="s">
         <v>109</v>
       </c>
@@ -1765,6 +1762,9 @@
       <c r="D6" t="s">
         <v>98</v>
       </c>
+      <c r="E6" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1779,6 +1779,9 @@
       <c r="D7" t="s">
         <v>99</v>
       </c>
+      <c r="E7" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1793,6 +1796,9 @@
       <c r="D8" t="s">
         <v>100</v>
       </c>
+      <c r="E8" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1807,6 +1813,9 @@
       <c r="D9" t="s">
         <v>101</v>
       </c>
+      <c r="E9" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1821,6 +1830,9 @@
       <c r="D10" t="s">
         <v>102</v>
       </c>
+      <c r="E10" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1835,6 +1847,9 @@
       <c r="D11" t="s">
         <v>18</v>
       </c>
+      <c r="E11" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1849,6 +1864,9 @@
       <c r="D12" t="s">
         <v>20</v>
       </c>
+      <c r="E12" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1863,6 +1881,9 @@
       <c r="D13" t="s">
         <v>22</v>
       </c>
+      <c r="E13" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1877,6 +1898,9 @@
       <c r="D14" t="s">
         <v>24</v>
       </c>
+      <c r="E14" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1891,6 +1915,9 @@
       <c r="D15" t="s">
         <v>26</v>
       </c>
+      <c r="E15" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1905,6 +1932,9 @@
       <c r="D16" t="s">
         <v>28</v>
       </c>
+      <c r="E16" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1919,6 +1949,9 @@
       <c r="D17" t="s">
         <v>30</v>
       </c>
+      <c r="E17" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1933,6 +1966,9 @@
       <c r="D18" t="s">
         <v>32</v>
       </c>
+      <c r="E18" s="5" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1946,6 +1982,9 @@
       </c>
       <c r="D19" t="s">
         <v>34</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -2522,7 +2561,7 @@
         <v>118</v>
       </c>
       <c r="B55" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C55" t="s">
         <v>126</v>
@@ -2531,7 +2570,7 @@
         <v>117</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2539,7 +2578,7 @@
         <v>118</v>
       </c>
       <c r="B56" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C56" t="s">
         <v>126</v>
@@ -2548,38 +2587,41 @@
         <v>117</v>
       </c>
       <c r="H56" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B57" s="6" t="s">
-        <v>196</v>
+        <v>121</v>
       </c>
       <c r="C57" t="s">
-        <v>126</v>
+        <v>130</v>
+      </c>
+      <c r="D57" t="s">
+        <v>122</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="H57" s="1" t="s">
-        <v>197</v>
+      <c r="F57" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B58" s="6" t="s">
-        <v>121</v>
+      <c r="A58" t="s">
+        <v>131</v>
+      </c>
+      <c r="B58" t="s">
+        <v>132</v>
       </c>
       <c r="C58" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="D58" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F58" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2587,16 +2629,19 @@
         <v>131</v>
       </c>
       <c r="B59" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C59" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
       <c r="D59" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E59" s="5" t="s">
         <v>120</v>
+      </c>
+      <c r="F59" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2604,13 +2649,13 @@
         <v>131</v>
       </c>
       <c r="B60" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C60" t="s">
         <v>135</v>
       </c>
       <c r="D60" t="s">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>120</v>
@@ -2624,13 +2669,13 @@
         <v>131</v>
       </c>
       <c r="B61" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C61" t="s">
         <v>135</v>
       </c>
       <c r="D61" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>120</v>
@@ -2644,13 +2689,13 @@
         <v>131</v>
       </c>
       <c r="B62" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C62" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D62" t="s">
-        <v>199</v>
+        <v>140</v>
       </c>
       <c r="E62" s="5" t="s">
         <v>120</v>
@@ -2661,16 +2706,16 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="B63" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
-      </c>
-      <c r="D63" t="s">
-        <v>140</v>
+        <v>135</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>198</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>120</v>
@@ -2684,19 +2729,16 @@
         <v>141</v>
       </c>
       <c r="B64" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C64" t="s">
         <v>135</v>
       </c>
-      <c r="D64" s="3" t="s">
-        <v>200</v>
+      <c r="D64" t="s">
+        <v>199</v>
       </c>
       <c r="E64" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F64" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2704,13 +2746,13 @@
         <v>141</v>
       </c>
       <c r="B65" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C65" t="s">
         <v>135</v>
       </c>
       <c r="D65" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>120</v>
@@ -2721,13 +2763,13 @@
         <v>141</v>
       </c>
       <c r="B66" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C66" t="s">
         <v>135</v>
       </c>
       <c r="D66" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E66" s="5" t="s">
         <v>120</v>
@@ -2738,16 +2780,13 @@
         <v>141</v>
       </c>
       <c r="B67" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C67" t="s">
         <v>135</v>
       </c>
       <c r="D67" t="s">
-        <v>203</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>120</v>
+        <v>202</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2755,13 +2794,13 @@
         <v>141</v>
       </c>
       <c r="B68" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="C68" t="s">
         <v>135</v>
       </c>
       <c r="D68" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2769,13 +2808,13 @@
         <v>141</v>
       </c>
       <c r="B69" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C69" t="s">
         <v>135</v>
       </c>
       <c r="D69" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2783,13 +2822,13 @@
         <v>141</v>
       </c>
       <c r="B70" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C70" t="s">
         <v>135</v>
       </c>
       <c r="D70" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2797,13 +2836,19 @@
         <v>141</v>
       </c>
       <c r="B71" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C71" t="s">
         <v>135</v>
       </c>
       <c r="D71" t="s">
-        <v>207</v>
+        <v>206</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F71" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2811,13 +2856,13 @@
         <v>141</v>
       </c>
       <c r="B72" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C72" t="s">
         <v>135</v>
       </c>
       <c r="D72" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>120</v>
@@ -2831,19 +2876,13 @@
         <v>141</v>
       </c>
       <c r="B73" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C73" t="s">
         <v>135</v>
       </c>
       <c r="D73" t="s">
-        <v>209</v>
-      </c>
-      <c r="E73" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F73" t="b">
-        <v>1</v>
+        <v>208</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2851,13 +2890,19 @@
         <v>141</v>
       </c>
       <c r="B74" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C74" t="s">
         <v>135</v>
       </c>
       <c r="D74" t="s">
-        <v>210</v>
+        <v>209</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F74" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2865,19 +2910,16 @@
         <v>141</v>
       </c>
       <c r="B75" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C75" t="s">
         <v>135</v>
       </c>
       <c r="D75" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E75" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F75" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2885,16 +2927,19 @@
         <v>141</v>
       </c>
       <c r="B76" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C76" t="s">
         <v>135</v>
       </c>
       <c r="D76" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E76" s="5" t="s">
         <v>120</v>
+      </c>
+      <c r="F76" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2902,13 +2947,13 @@
         <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C77" t="s">
         <v>135</v>
       </c>
       <c r="D77" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E77" s="5" t="s">
         <v>120</v>
@@ -2919,22 +2964,16 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="B78" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="C78" t="s">
         <v>135</v>
       </c>
       <c r="D78" t="s">
-        <v>214</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F78" t="b">
-        <v>1</v>
+        <v>136</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2942,13 +2981,19 @@
         <v>156</v>
       </c>
       <c r="B79" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C79" t="s">
         <v>135</v>
       </c>
       <c r="D79" t="s">
-        <v>136</v>
+        <v>213</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F79" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2956,19 +3001,13 @@
         <v>156</v>
       </c>
       <c r="B80" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C80" t="s">
         <v>135</v>
       </c>
       <c r="D80" t="s">
-        <v>215</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F80" t="b">
-        <v>1</v>
+        <v>214</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -2976,13 +3015,13 @@
         <v>156</v>
       </c>
       <c r="B81" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C81" t="s">
         <v>135</v>
       </c>
       <c r="D81" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -2990,13 +3029,13 @@
         <v>156</v>
       </c>
       <c r="B82" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C82" t="s">
         <v>135</v>
       </c>
       <c r="D82" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
@@ -3004,13 +3043,13 @@
         <v>156</v>
       </c>
       <c r="B83" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C83" t="s">
         <v>135</v>
       </c>
       <c r="D83" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
@@ -3018,13 +3057,19 @@
         <v>156</v>
       </c>
       <c r="B84" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C84" t="s">
         <v>135</v>
       </c>
       <c r="D84" t="s">
-        <v>219</v>
+        <v>218</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F84" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
@@ -3032,19 +3077,13 @@
         <v>156</v>
       </c>
       <c r="B85" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C85" t="s">
         <v>135</v>
       </c>
       <c r="D85" t="s">
-        <v>220</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F85" t="b">
-        <v>1</v>
+        <v>219</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -3052,13 +3091,19 @@
         <v>156</v>
       </c>
       <c r="B86" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C86" t="s">
         <v>135</v>
       </c>
       <c r="D86" t="s">
-        <v>221</v>
+        <v>220</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F86" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
@@ -3066,19 +3111,16 @@
         <v>156</v>
       </c>
       <c r="B87" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C87" t="s">
         <v>135</v>
       </c>
       <c r="D87" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F87" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -3086,16 +3128,19 @@
         <v>156</v>
       </c>
       <c r="B88" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C88" t="s">
         <v>135</v>
       </c>
       <c r="D88" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>120</v>
+      </c>
+      <c r="F88" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -3103,13 +3148,13 @@
         <v>156</v>
       </c>
       <c r="B89" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C89" t="s">
         <v>135</v>
       </c>
       <c r="D89" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>120</v>
@@ -3123,13 +3168,13 @@
         <v>156</v>
       </c>
       <c r="B90" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C90" t="s">
         <v>135</v>
       </c>
       <c r="D90" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>120</v>
@@ -3143,19 +3188,13 @@
         <v>156</v>
       </c>
       <c r="B91" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C91" t="s">
         <v>135</v>
       </c>
       <c r="D91" t="s">
-        <v>226</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F91" t="b">
-        <v>1</v>
+        <v>225</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
@@ -3163,13 +3202,13 @@
         <v>156</v>
       </c>
       <c r="B92" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C92" t="s">
         <v>135</v>
       </c>
       <c r="D92" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
@@ -3177,13 +3216,13 @@
         <v>156</v>
       </c>
       <c r="B93" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C93" t="s">
         <v>135</v>
       </c>
       <c r="D93" t="s">
-        <v>228</v>
+        <v>140</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
@@ -3191,32 +3230,35 @@
         <v>156</v>
       </c>
       <c r="B94" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C94" t="s">
         <v>135</v>
       </c>
       <c r="D94" t="s">
-        <v>140</v>
+        <v>227</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F94" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>156</v>
+        <v>193</v>
       </c>
       <c r="B95" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="C95" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D95" t="s">
-        <v>229</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F95" t="b">
+        <v>175</v>
+      </c>
+      <c r="G95" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3225,16 +3267,13 @@
         <v>193</v>
       </c>
       <c r="B96" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C96" t="s">
-        <v>130</v>
+        <v>93</v>
       </c>
       <c r="D96" t="s">
-        <v>175</v>
-      </c>
-      <c r="G96" t="b">
-        <v>1</v>
+        <v>176</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3242,13 +3281,13 @@
         <v>193</v>
       </c>
       <c r="B97" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C97" t="s">
-        <v>93</v>
+        <v>4</v>
       </c>
       <c r="D97" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
@@ -3256,13 +3295,16 @@
         <v>193</v>
       </c>
       <c r="B98" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C98" t="s">
-        <v>4</v>
+        <v>135</v>
       </c>
       <c r="D98" t="s">
-        <v>177</v>
+        <v>228</v>
+      </c>
+      <c r="G98" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -3270,13 +3312,13 @@
         <v>193</v>
       </c>
       <c r="B99" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C99" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="D99" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G99" t="b">
         <v>1</v>
@@ -3287,13 +3329,13 @@
         <v>193</v>
       </c>
       <c r="B100" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C100" t="s">
         <v>130</v>
       </c>
       <c r="D100" t="s">
-        <v>231</v>
+        <v>178</v>
       </c>
       <c r="G100" t="b">
         <v>1</v>
@@ -3304,16 +3346,13 @@
         <v>193</v>
       </c>
       <c r="B101" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C101" t="s">
-        <v>130</v>
+        <v>4</v>
       </c>
       <c r="D101" t="s">
-        <v>178</v>
-      </c>
-      <c r="G101" t="b">
-        <v>1</v>
+        <v>179</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
@@ -3321,13 +3360,19 @@
         <v>193</v>
       </c>
       <c r="B102" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C102" t="s">
         <v>4</v>
       </c>
       <c r="D102" t="s">
-        <v>179</v>
+        <v>180</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="H102" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -3335,19 +3380,19 @@
         <v>193</v>
       </c>
       <c r="B103" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C103" t="s">
-        <v>4</v>
+        <v>130</v>
       </c>
       <c r="D103" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E103" s="5" t="s">
         <v>119</v>
       </c>
       <c r="H103" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -3355,35 +3400,15 @@
         <v>193</v>
       </c>
       <c r="B104" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="C104" t="s">
-        <v>130</v>
+        <v>4</v>
       </c>
       <c r="D104" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="H104" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>193</v>
-      </c>
-      <c r="B105" t="s">
-        <v>184</v>
-      </c>
-      <c r="C105" t="s">
-        <v>4</v>
-      </c>
-      <c r="D105" t="s">
-        <v>182</v>
-      </c>
-      <c r="E105" s="5" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Optimised and got yearly input working
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0348AC0-FD8C-4A53-AB52-84701DE9209E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D32D6B7-BC49-4D90-B195-08105063FC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="241">
   <si>
     <t>type</t>
   </si>
@@ -739,6 +739,24 @@
   </si>
   <si>
     <t>We will need to parse these a list</t>
+  </si>
+  <si>
+    <t>VRGBPE</t>
+  </si>
+  <si>
+    <t>ERGBPE</t>
+  </si>
+  <si>
+    <t>SRGBPE</t>
+  </si>
+  <si>
+    <t>ERNE</t>
+  </si>
+  <si>
+    <t>LRGBPS</t>
+  </si>
+  <si>
+    <t>_RGBPS</t>
   </si>
 </sst>
 </file>
@@ -2623,6 +2641,9 @@
       <c r="E58" s="5" t="s">
         <v>120</v>
       </c>
+      <c r="G58" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">

</xml_diff>

<commit_message>
Excellent full run-through, database derived
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D32D6B7-BC49-4D90-B195-08105063FC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA81397A-8152-4731-99BD-619AA57E2897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="235">
   <si>
     <t>type</t>
   </si>
@@ -739,24 +739,6 @@
   </si>
   <si>
     <t>We will need to parse these a list</t>
-  </si>
-  <si>
-    <t>VRGBPE</t>
-  </si>
-  <si>
-    <t>ERGBPE</t>
-  </si>
-  <si>
-    <t>SRGBPE</t>
-  </si>
-  <si>
-    <t>ERNE</t>
-  </si>
-  <si>
-    <t>LRGBPS</t>
-  </si>
-  <si>
-    <t>_RGBPS</t>
   </si>
 </sst>
 </file>
@@ -2392,6 +2374,9 @@
       <c r="D42" t="s">
         <v>79</v>
       </c>
+      <c r="G42" t="b">
+        <v>1</v>
+      </c>
       <c r="I42" s="7"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -2664,6 +2649,9 @@
       <c r="F59" t="b">
         <v>1</v>
       </c>
+      <c r="G59" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -2684,6 +2672,9 @@
       <c r="F60" t="b">
         <v>1</v>
       </c>
+      <c r="G60" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
@@ -2704,6 +2695,9 @@
       <c r="F61" t="b">
         <v>1</v>
       </c>
+      <c r="G61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -2722,6 +2716,9 @@
         <v>120</v>
       </c>
       <c r="F62" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Set up ready to deflate variables
</commit_message>
<xml_diff>
--- a/build/input/raw_properties.xlsx
+++ b/build/input/raw_properties.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazyst\Files\ucl\Dissertation\build\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazym\Documents\Code\dissertation\build\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA81397A-8152-4731-99BD-619AA57E2897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57592CB4-7882-4C27-AFB2-1472BBA85D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
+    <workbookView xWindow="-17295" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{016D8697-EE21-4866-BE68-DA78E4F0384A}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_properties" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="238">
   <si>
     <t>type</t>
   </si>
@@ -739,6 +739,15 @@
   </si>
   <si>
     <t>We will need to parse these a list</t>
+  </si>
+  <si>
+    <t>deflate</t>
+  </si>
+  <si>
+    <t>gdpdef</t>
+  </si>
+  <si>
+    <t>cpih</t>
   </si>
 </sst>
 </file>
@@ -1626,18 +1635,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0009E10-3834-4149-8D15-4D105A1770B9}">
-  <dimension ref="A1:I104"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J104"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="38.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="38.7265625" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="5"/>
-    <col min="13" max="13" width="43.85546875" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="5"/>
+    <col min="14" max="14" width="43.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
@@ -1660,10 +1669,13 @@
         <v>230</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1682,11 +1694,11 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>118</v>
       </c>
@@ -1709,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1725,11 +1737,11 @@
       <c r="E4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1745,11 +1757,11 @@
       <c r="E5" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1766,7 +1778,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1783,7 +1795,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1800,7 +1812,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1817,7 +1829,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1834,7 +1846,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1851,7 +1863,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1868,7 +1880,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1885,7 +1897,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -1902,7 +1914,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -1919,7 +1931,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1936,7 +1948,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1953,7 +1965,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -1970,7 +1982,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -1987,7 +1999,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -2001,7 +2013,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>2</v>
       </c>
@@ -2015,7 +2027,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -2029,7 +2041,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>2</v>
       </c>
@@ -2048,11 +2060,11 @@
       <c r="F23" t="b">
         <v>0</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -2072,7 +2084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>2</v>
       </c>
@@ -2092,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -2108,11 +2120,11 @@
       <c r="G26" t="b">
         <v>1</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>2</v>
       </c>
@@ -2131,11 +2143,11 @@
       <c r="F27" t="b">
         <v>1</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -2149,7 +2161,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>2</v>
       </c>
@@ -2168,11 +2180,11 @@
       <c r="F29" t="b">
         <v>1</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -2192,7 +2204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -2206,7 +2218,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -2219,14 +2231,14 @@
       <c r="D32" t="s">
         <v>60</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="I32" s="7" t="s">
+      <c r="J32" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -2239,9 +2251,9 @@
       <c r="D33" t="s">
         <v>62</v>
       </c>
-      <c r="I33" s="7"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="7"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -2254,9 +2266,9 @@
       <c r="D34" t="s">
         <v>64</v>
       </c>
-      <c r="I34" s="7"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="7"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -2269,9 +2281,9 @@
       <c r="D35" t="s">
         <v>66</v>
       </c>
-      <c r="I35" s="7"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="7"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>2</v>
       </c>
@@ -2284,9 +2296,9 @@
       <c r="D36" t="s">
         <v>68</v>
       </c>
-      <c r="I36" s="7"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="7"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -2299,9 +2311,9 @@
       <c r="D37" t="s">
         <v>70</v>
       </c>
-      <c r="I37" s="7"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" s="7"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -2314,9 +2326,9 @@
       <c r="D38" t="s">
         <v>72</v>
       </c>
-      <c r="I38" s="7"/>
-    </row>
-    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="J38" s="7"/>
+    </row>
+    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -2329,9 +2341,9 @@
       <c r="D39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="I39" s="7"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" s="7"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -2344,9 +2356,9 @@
       <c r="D40" t="s">
         <v>75</v>
       </c>
-      <c r="I40" s="7"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" s="7"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -2359,9 +2371,9 @@
       <c r="D41" t="s">
         <v>77</v>
       </c>
-      <c r="I41" s="7"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" s="7"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>2</v>
       </c>
@@ -2377,9 +2389,9 @@
       <c r="G42" t="b">
         <v>1</v>
       </c>
-      <c r="I42" s="7"/>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" s="7"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>2</v>
       </c>
@@ -2392,9 +2404,9 @@
       <c r="D43" t="s">
         <v>81</v>
       </c>
-      <c r="I43" s="7"/>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" s="7"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -2407,9 +2419,9 @@
       <c r="D44" t="s">
         <v>83</v>
       </c>
-      <c r="I44" s="7"/>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" s="7"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>2</v>
       </c>
@@ -2422,9 +2434,9 @@
       <c r="D45" t="s">
         <v>85</v>
       </c>
-      <c r="I45" s="7"/>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" s="7"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>2</v>
       </c>
@@ -2437,9 +2449,9 @@
       <c r="D46" t="s">
         <v>87</v>
       </c>
-      <c r="I46" s="7"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" s="7"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>2</v>
       </c>
@@ -2452,9 +2464,9 @@
       <c r="D47" t="s">
         <v>89</v>
       </c>
-      <c r="I47" s="7"/>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" s="7"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>2</v>
       </c>
@@ -2467,9 +2479,9 @@
       <c r="D48" t="s">
         <v>91</v>
       </c>
-      <c r="I48" s="7"/>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J48" s="7"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>2</v>
       </c>
@@ -2489,7 +2501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -2512,7 +2524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>123</v>
       </c>
@@ -2522,11 +2534,11 @@
       <c r="E51" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="H51" t="s">
+      <c r="I51" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>124</v>
       </c>
@@ -2537,7 +2549,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>107</v>
       </c>
@@ -2548,7 +2560,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>128</v>
       </c>
@@ -2559,7 +2571,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>118</v>
       </c>
@@ -2572,11 +2584,11 @@
       <c r="E55" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="I55" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>118</v>
       </c>
@@ -2589,11 +2601,11 @@
       <c r="E56" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="H56" t="s">
+      <c r="I56" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B57" s="6" t="s">
         <v>121</v>
       </c>
@@ -2610,7 +2622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>131</v>
       </c>
@@ -2630,7 +2642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>131</v>
       </c>
@@ -2652,8 +2664,11 @@
       <c r="G59" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H59" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>131</v>
       </c>
@@ -2675,8 +2690,11 @@
       <c r="G60" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H60" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>131</v>
       </c>
@@ -2698,8 +2716,11 @@
       <c r="G61" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H61" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>131</v>
       </c>
@@ -2721,8 +2742,9 @@
       <c r="G62" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>141</v>
       </c>
@@ -2741,8 +2763,11 @@
       <c r="F63" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H63" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>141</v>
       </c>
@@ -2758,8 +2783,11 @@
       <c r="E64" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H64" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>141</v>
       </c>
@@ -2775,8 +2803,11 @@
       <c r="E65" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H65" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>141</v>
       </c>
@@ -2792,8 +2823,11 @@
       <c r="E66" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H66" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>141</v>
       </c>
@@ -2806,8 +2840,11 @@
       <c r="D67" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H67" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>141</v>
       </c>
@@ -2820,8 +2857,11 @@
       <c r="D68" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H68" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>141</v>
       </c>
@@ -2834,8 +2874,11 @@
       <c r="D69" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H69" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>141</v>
       </c>
@@ -2848,8 +2891,11 @@
       <c r="D70" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H70" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>141</v>
       </c>
@@ -2868,8 +2914,11 @@
       <c r="F71" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H71" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>141</v>
       </c>
@@ -2888,8 +2937,11 @@
       <c r="F72" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H72" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>141</v>
       </c>
@@ -2902,8 +2954,11 @@
       <c r="D73" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H73" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>141</v>
       </c>
@@ -2922,8 +2977,11 @@
       <c r="F74" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H74" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>141</v>
       </c>
@@ -2939,8 +2997,11 @@
       <c r="E75" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H75" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>141</v>
       </c>
@@ -2959,8 +3020,11 @@
       <c r="F76" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H76" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>141</v>
       </c>
@@ -2979,8 +3043,11 @@
       <c r="F77" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H77" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>156</v>
       </c>
@@ -2993,8 +3060,11 @@
       <c r="D78" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H78" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>156</v>
       </c>
@@ -3013,8 +3083,11 @@
       <c r="F79" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H79" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>156</v>
       </c>
@@ -3027,8 +3100,11 @@
       <c r="D80" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H80" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>156</v>
       </c>
@@ -3041,8 +3117,11 @@
       <c r="D81" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H81" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>156</v>
       </c>
@@ -3055,8 +3134,11 @@
       <c r="D82" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H82" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>156</v>
       </c>
@@ -3069,8 +3151,11 @@
       <c r="D83" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H83" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>156</v>
       </c>
@@ -3089,8 +3174,11 @@
       <c r="F84" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H84" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>156</v>
       </c>
@@ -3103,8 +3191,11 @@
       <c r="D85" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H85" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>156</v>
       </c>
@@ -3123,8 +3214,11 @@
       <c r="F86" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H86" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>156</v>
       </c>
@@ -3140,8 +3234,11 @@
       <c r="E87" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H87" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>156</v>
       </c>
@@ -3160,8 +3257,11 @@
       <c r="F88" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H88" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>156</v>
       </c>
@@ -3180,8 +3280,11 @@
       <c r="F89" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H89" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>156</v>
       </c>
@@ -3200,8 +3303,11 @@
       <c r="F90" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H90" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>156</v>
       </c>
@@ -3214,8 +3320,11 @@
       <c r="D91" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H91" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>156</v>
       </c>
@@ -3228,8 +3337,11 @@
       <c r="D92" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H92" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -3242,8 +3354,9 @@
       <c r="D93" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H93" s="5"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>156</v>
       </c>
@@ -3262,8 +3375,11 @@
       <c r="F94" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H94" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>193</v>
       </c>
@@ -3280,7 +3396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>193</v>
       </c>
@@ -3294,7 +3410,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>193</v>
       </c>
@@ -3308,7 +3424,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>193</v>
       </c>
@@ -3325,7 +3441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>193</v>
       </c>
@@ -3342,7 +3458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>193</v>
       </c>
@@ -3359,7 +3475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>193</v>
       </c>
@@ -3373,7 +3489,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>193</v>
       </c>
@@ -3389,11 +3505,11 @@
       <c r="E102" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H102" t="s">
+      <c r="I102" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>193</v>
       </c>
@@ -3409,11 +3525,11 @@
       <c r="E103" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="H103" t="s">
+      <c r="I103" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>193</v>
       </c>
@@ -3432,7 +3548,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I32:I48"/>
+    <mergeCell ref="J32:J48"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>